<commit_message>
gender addition to new db
</commit_message>
<xml_diff>
--- a/public/assets/templates/cliniq-patient-account-import.xlsx
+++ b/public/assets/templates/cliniq-patient-account-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patient Accounts" sheetId="1" r:id="R5f81c87942d74c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Raa583a6d832846cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patient Accounts" sheetId="1" r:id="Rd9c28c8d59ff459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R6a818c15a5a64578"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,7 +52,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -74,8 +74,23 @@
         <x:fgColor rgb="FFE8F6EC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23422C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F6EC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="19">
     <x:border/>
     <x:border>
       <x:right style="thin">
@@ -185,11 +200,47 @@
         <x:color rgb="FFE8D99A"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF4E6756"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF4E6756"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF4E6756"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF4E6756"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8D99A"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFE8D99A"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8D99A"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE8D99A"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE8D99A"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8D99A"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="74">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -297,6 +348,35 @@
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -505,10 +585,11 @@
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="32" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -531,15 +612,18 @@
         <x:v>Birthdate</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
+        <x:v>Sex</x:v>
+      </x:c>
+      <x:c r="H1" s="10" t="str">
         <x:v>Program Code / Department Code</x:v>
       </x:c>
-      <x:c r="H1" s="10" t="str">
+      <x:c r="I1" s="10" t="str">
         <x:v>Year Level / Employment Type</x:v>
       </x:c>
-      <x:c r="I1" s="10" t="str">
+      <x:c r="J1" s="11" t="str">
         <x:v>Section Code / Title / Position</x:v>
       </x:c>
-      <x:c r="J1" s="11" t="str">
+      <x:c r="K1" s="61" t="str">
         <x:v>Academic Year</x:v>
       </x:c>
     </x:row>
@@ -550,10 +634,11 @@
       <x:c r="D2" s="14"/>
       <x:c r="E2" s="14"/>
       <x:c r="F2" s="20"/>
-      <x:c r="G2" s="14"/>
+      <x:c r="G2" s="17"/>
       <x:c r="H2" s="14"/>
       <x:c r="I2" s="14"/>
       <x:c r="J2" s="14"/>
+      <x:c r="K2" s="63"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="18"/>
@@ -562,10 +647,11 @@
       <x:c r="D3" s="15"/>
       <x:c r="E3" s="15"/>
       <x:c r="F3" s="21"/>
-      <x:c r="G3" s="15"/>
+      <x:c r="G3" s="18"/>
       <x:c r="H3" s="15"/>
       <x:c r="I3" s="15"/>
       <x:c r="J3" s="15"/>
+      <x:c r="K3" s="64"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18"/>
@@ -574,10 +660,11 @@
       <x:c r="D4" s="15"/>
       <x:c r="E4" s="15"/>
       <x:c r="F4" s="21"/>
-      <x:c r="G4" s="15"/>
+      <x:c r="G4" s="18"/>
       <x:c r="H4" s="15"/>
       <x:c r="I4" s="15"/>
       <x:c r="J4" s="15"/>
+      <x:c r="K4" s="64"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="18"/>
@@ -586,10 +673,11 @@
       <x:c r="D5" s="15"/>
       <x:c r="E5" s="15"/>
       <x:c r="F5" s="21"/>
-      <x:c r="G5" s="15"/>
+      <x:c r="G5" s="18"/>
       <x:c r="H5" s="15"/>
       <x:c r="I5" s="15"/>
       <x:c r="J5" s="15"/>
+      <x:c r="K5" s="64"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="18"/>
@@ -598,10 +686,11 @@
       <x:c r="D6" s="15"/>
       <x:c r="E6" s="15"/>
       <x:c r="F6" s="21"/>
-      <x:c r="G6" s="15"/>
+      <x:c r="G6" s="18"/>
       <x:c r="H6" s="15"/>
       <x:c r="I6" s="15"/>
       <x:c r="J6" s="15"/>
+      <x:c r="K6" s="64"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="18"/>
@@ -610,10 +699,11 @@
       <x:c r="D7" s="15"/>
       <x:c r="E7" s="15"/>
       <x:c r="F7" s="21"/>
-      <x:c r="G7" s="15"/>
+      <x:c r="G7" s="18"/>
       <x:c r="H7" s="15"/>
       <x:c r="I7" s="15"/>
       <x:c r="J7" s="15"/>
+      <x:c r="K7" s="64"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="18"/>
@@ -622,10 +712,11 @@
       <x:c r="D8" s="15"/>
       <x:c r="E8" s="15"/>
       <x:c r="F8" s="21"/>
-      <x:c r="G8" s="15"/>
+      <x:c r="G8" s="18"/>
       <x:c r="H8" s="15"/>
       <x:c r="I8" s="15"/>
       <x:c r="J8" s="15"/>
+      <x:c r="K8" s="64"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="18"/>
@@ -634,10 +725,11 @@
       <x:c r="D9" s="15"/>
       <x:c r="E9" s="15"/>
       <x:c r="F9" s="21"/>
-      <x:c r="G9" s="15"/>
+      <x:c r="G9" s="18"/>
       <x:c r="H9" s="15"/>
       <x:c r="I9" s="15"/>
       <x:c r="J9" s="15"/>
+      <x:c r="K9" s="64"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="18"/>
@@ -646,10 +738,11 @@
       <x:c r="D10" s="15"/>
       <x:c r="E10" s="15"/>
       <x:c r="F10" s="21"/>
-      <x:c r="G10" s="15"/>
+      <x:c r="G10" s="18"/>
       <x:c r="H10" s="15"/>
       <x:c r="I10" s="15"/>
       <x:c r="J10" s="15"/>
+      <x:c r="K10" s="64"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18"/>
@@ -658,10 +751,11 @@
       <x:c r="D11" s="15"/>
       <x:c r="E11" s="15"/>
       <x:c r="F11" s="21"/>
-      <x:c r="G11" s="15"/>
+      <x:c r="G11" s="18"/>
       <x:c r="H11" s="15"/>
       <x:c r="I11" s="15"/>
       <x:c r="J11" s="15"/>
+      <x:c r="K11" s="64"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="18"/>
@@ -670,10 +764,11 @@
       <x:c r="D12" s="15"/>
       <x:c r="E12" s="15"/>
       <x:c r="F12" s="21"/>
-      <x:c r="G12" s="15"/>
+      <x:c r="G12" s="18"/>
       <x:c r="H12" s="15"/>
       <x:c r="I12" s="15"/>
       <x:c r="J12" s="15"/>
+      <x:c r="K12" s="64"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="18"/>
@@ -682,10 +777,11 @@
       <x:c r="D13" s="15"/>
       <x:c r="E13" s="15"/>
       <x:c r="F13" s="21"/>
-      <x:c r="G13" s="15"/>
+      <x:c r="G13" s="18"/>
       <x:c r="H13" s="15"/>
       <x:c r="I13" s="15"/>
       <x:c r="J13" s="15"/>
+      <x:c r="K13" s="64"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="18"/>
@@ -694,10 +790,11 @@
       <x:c r="D14" s="15"/>
       <x:c r="E14" s="15"/>
       <x:c r="F14" s="21"/>
-      <x:c r="G14" s="15"/>
+      <x:c r="G14" s="18"/>
       <x:c r="H14" s="15"/>
       <x:c r="I14" s="15"/>
       <x:c r="J14" s="15"/>
+      <x:c r="K14" s="64"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="18"/>
@@ -706,10 +803,11 @@
       <x:c r="D15" s="15"/>
       <x:c r="E15" s="15"/>
       <x:c r="F15" s="21"/>
-      <x:c r="G15" s="15"/>
+      <x:c r="G15" s="18"/>
       <x:c r="H15" s="15"/>
       <x:c r="I15" s="15"/>
       <x:c r="J15" s="15"/>
+      <x:c r="K15" s="64"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="18"/>
@@ -718,10 +816,11 @@
       <x:c r="D16" s="15"/>
       <x:c r="E16" s="15"/>
       <x:c r="F16" s="21"/>
-      <x:c r="G16" s="15"/>
+      <x:c r="G16" s="18"/>
       <x:c r="H16" s="15"/>
       <x:c r="I16" s="15"/>
       <x:c r="J16" s="15"/>
+      <x:c r="K16" s="64"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="18"/>
@@ -730,10 +829,11 @@
       <x:c r="D17" s="15"/>
       <x:c r="E17" s="15"/>
       <x:c r="F17" s="21"/>
-      <x:c r="G17" s="15"/>
+      <x:c r="G17" s="18"/>
       <x:c r="H17" s="15"/>
       <x:c r="I17" s="15"/>
       <x:c r="J17" s="15"/>
+      <x:c r="K17" s="64"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="18"/>
@@ -742,10 +842,11 @@
       <x:c r="D18" s="15"/>
       <x:c r="E18" s="15"/>
       <x:c r="F18" s="21"/>
-      <x:c r="G18" s="15"/>
+      <x:c r="G18" s="18"/>
       <x:c r="H18" s="15"/>
       <x:c r="I18" s="15"/>
       <x:c r="J18" s="15"/>
+      <x:c r="K18" s="64"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="18"/>
@@ -754,10 +855,11 @@
       <x:c r="D19" s="15"/>
       <x:c r="E19" s="15"/>
       <x:c r="F19" s="21"/>
-      <x:c r="G19" s="15"/>
+      <x:c r="G19" s="18"/>
       <x:c r="H19" s="15"/>
       <x:c r="I19" s="15"/>
       <x:c r="J19" s="15"/>
+      <x:c r="K19" s="64"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="18"/>
@@ -766,10 +868,11 @@
       <x:c r="D20" s="15"/>
       <x:c r="E20" s="15"/>
       <x:c r="F20" s="21"/>
-      <x:c r="G20" s="15"/>
+      <x:c r="G20" s="18"/>
       <x:c r="H20" s="15"/>
       <x:c r="I20" s="15"/>
       <x:c r="J20" s="15"/>
+      <x:c r="K20" s="64"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="18"/>
@@ -778,10 +881,11 @@
       <x:c r="D21" s="15"/>
       <x:c r="E21" s="15"/>
       <x:c r="F21" s="21"/>
-      <x:c r="G21" s="15"/>
+      <x:c r="G21" s="18"/>
       <x:c r="H21" s="15"/>
       <x:c r="I21" s="15"/>
       <x:c r="J21" s="15"/>
+      <x:c r="K21" s="64"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="18"/>
@@ -790,10 +894,11 @@
       <x:c r="D22" s="15"/>
       <x:c r="E22" s="15"/>
       <x:c r="F22" s="21"/>
-      <x:c r="G22" s="15"/>
+      <x:c r="G22" s="18"/>
       <x:c r="H22" s="15"/>
       <x:c r="I22" s="15"/>
       <x:c r="J22" s="15"/>
+      <x:c r="K22" s="64"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="18"/>
@@ -802,10 +907,11 @@
       <x:c r="D23" s="15"/>
       <x:c r="E23" s="15"/>
       <x:c r="F23" s="21"/>
-      <x:c r="G23" s="15"/>
+      <x:c r="G23" s="18"/>
       <x:c r="H23" s="15"/>
       <x:c r="I23" s="15"/>
       <x:c r="J23" s="15"/>
+      <x:c r="K23" s="64"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="18"/>
@@ -814,10 +920,11 @@
       <x:c r="D24" s="15"/>
       <x:c r="E24" s="15"/>
       <x:c r="F24" s="21"/>
-      <x:c r="G24" s="15"/>
+      <x:c r="G24" s="18"/>
       <x:c r="H24" s="15"/>
       <x:c r="I24" s="15"/>
       <x:c r="J24" s="15"/>
+      <x:c r="K24" s="64"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18"/>
@@ -826,10 +933,11 @@
       <x:c r="D25" s="15"/>
       <x:c r="E25" s="15"/>
       <x:c r="F25" s="21"/>
-      <x:c r="G25" s="15"/>
+      <x:c r="G25" s="18"/>
       <x:c r="H25" s="15"/>
       <x:c r="I25" s="15"/>
       <x:c r="J25" s="15"/>
+      <x:c r="K25" s="64"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="18"/>
@@ -838,10 +946,11 @@
       <x:c r="D26" s="15"/>
       <x:c r="E26" s="15"/>
       <x:c r="F26" s="21"/>
-      <x:c r="G26" s="15"/>
+      <x:c r="G26" s="18"/>
       <x:c r="H26" s="15"/>
       <x:c r="I26" s="15"/>
       <x:c r="J26" s="15"/>
+      <x:c r="K26" s="64"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="18"/>
@@ -850,10 +959,11 @@
       <x:c r="D27" s="15"/>
       <x:c r="E27" s="15"/>
       <x:c r="F27" s="21"/>
-      <x:c r="G27" s="15"/>
+      <x:c r="G27" s="18"/>
       <x:c r="H27" s="15"/>
       <x:c r="I27" s="15"/>
       <x:c r="J27" s="15"/>
+      <x:c r="K27" s="64"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="18"/>
@@ -862,10 +972,11 @@
       <x:c r="D28" s="15"/>
       <x:c r="E28" s="15"/>
       <x:c r="F28" s="21"/>
-      <x:c r="G28" s="15"/>
+      <x:c r="G28" s="18"/>
       <x:c r="H28" s="15"/>
       <x:c r="I28" s="15"/>
       <x:c r="J28" s="15"/>
+      <x:c r="K28" s="64"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="18"/>
@@ -874,10 +985,11 @@
       <x:c r="D29" s="15"/>
       <x:c r="E29" s="15"/>
       <x:c r="F29" s="21"/>
-      <x:c r="G29" s="15"/>
+      <x:c r="G29" s="18"/>
       <x:c r="H29" s="15"/>
       <x:c r="I29" s="15"/>
       <x:c r="J29" s="15"/>
+      <x:c r="K29" s="64"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="18"/>
@@ -886,10 +998,11 @@
       <x:c r="D30" s="15"/>
       <x:c r="E30" s="15"/>
       <x:c r="F30" s="21"/>
-      <x:c r="G30" s="15"/>
+      <x:c r="G30" s="18"/>
       <x:c r="H30" s="15"/>
       <x:c r="I30" s="15"/>
       <x:c r="J30" s="15"/>
+      <x:c r="K30" s="64"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="18"/>
@@ -898,10 +1011,11 @@
       <x:c r="D31" s="15"/>
       <x:c r="E31" s="15"/>
       <x:c r="F31" s="21"/>
-      <x:c r="G31" s="15"/>
+      <x:c r="G31" s="18"/>
       <x:c r="H31" s="15"/>
       <x:c r="I31" s="15"/>
       <x:c r="J31" s="15"/>
+      <x:c r="K31" s="64"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="18"/>
@@ -910,10 +1024,11 @@
       <x:c r="D32" s="15"/>
       <x:c r="E32" s="15"/>
       <x:c r="F32" s="21"/>
-      <x:c r="G32" s="15"/>
+      <x:c r="G32" s="18"/>
       <x:c r="H32" s="15"/>
       <x:c r="I32" s="15"/>
       <x:c r="J32" s="15"/>
+      <x:c r="K32" s="64"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="18"/>
@@ -922,10 +1037,11 @@
       <x:c r="D33" s="15"/>
       <x:c r="E33" s="15"/>
       <x:c r="F33" s="21"/>
-      <x:c r="G33" s="15"/>
+      <x:c r="G33" s="18"/>
       <x:c r="H33" s="15"/>
       <x:c r="I33" s="15"/>
       <x:c r="J33" s="15"/>
+      <x:c r="K33" s="64"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="18"/>
@@ -934,10 +1050,11 @@
       <x:c r="D34" s="15"/>
       <x:c r="E34" s="15"/>
       <x:c r="F34" s="21"/>
-      <x:c r="G34" s="15"/>
+      <x:c r="G34" s="18"/>
       <x:c r="H34" s="15"/>
       <x:c r="I34" s="15"/>
       <x:c r="J34" s="15"/>
+      <x:c r="K34" s="64"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="18"/>
@@ -946,10 +1063,11 @@
       <x:c r="D35" s="15"/>
       <x:c r="E35" s="15"/>
       <x:c r="F35" s="21"/>
-      <x:c r="G35" s="15"/>
+      <x:c r="G35" s="18"/>
       <x:c r="H35" s="15"/>
       <x:c r="I35" s="15"/>
       <x:c r="J35" s="15"/>
+      <x:c r="K35" s="64"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="18"/>
@@ -958,10 +1076,11 @@
       <x:c r="D36" s="15"/>
       <x:c r="E36" s="15"/>
       <x:c r="F36" s="21"/>
-      <x:c r="G36" s="15"/>
+      <x:c r="G36" s="18"/>
       <x:c r="H36" s="15"/>
       <x:c r="I36" s="15"/>
       <x:c r="J36" s="15"/>
+      <x:c r="K36" s="64"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="18"/>
@@ -970,10 +1089,11 @@
       <x:c r="D37" s="15"/>
       <x:c r="E37" s="15"/>
       <x:c r="F37" s="21"/>
-      <x:c r="G37" s="15"/>
+      <x:c r="G37" s="18"/>
       <x:c r="H37" s="15"/>
       <x:c r="I37" s="15"/>
       <x:c r="J37" s="15"/>
+      <x:c r="K37" s="64"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="18"/>
@@ -982,10 +1102,11 @@
       <x:c r="D38" s="15"/>
       <x:c r="E38" s="15"/>
       <x:c r="F38" s="21"/>
-      <x:c r="G38" s="15"/>
+      <x:c r="G38" s="18"/>
       <x:c r="H38" s="15"/>
       <x:c r="I38" s="15"/>
       <x:c r="J38" s="15"/>
+      <x:c r="K38" s="64"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="18"/>
@@ -994,10 +1115,11 @@
       <x:c r="D39" s="15"/>
       <x:c r="E39" s="15"/>
       <x:c r="F39" s="21"/>
-      <x:c r="G39" s="15"/>
+      <x:c r="G39" s="18"/>
       <x:c r="H39" s="15"/>
       <x:c r="I39" s="15"/>
       <x:c r="J39" s="15"/>
+      <x:c r="K39" s="64"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="18"/>
@@ -1006,10 +1128,11 @@
       <x:c r="D40" s="15"/>
       <x:c r="E40" s="15"/>
       <x:c r="F40" s="21"/>
-      <x:c r="G40" s="15"/>
+      <x:c r="G40" s="18"/>
       <x:c r="H40" s="15"/>
       <x:c r="I40" s="15"/>
       <x:c r="J40" s="15"/>
+      <x:c r="K40" s="64"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="18"/>
@@ -1018,10 +1141,11 @@
       <x:c r="D41" s="15"/>
       <x:c r="E41" s="15"/>
       <x:c r="F41" s="21"/>
-      <x:c r="G41" s="15"/>
+      <x:c r="G41" s="18"/>
       <x:c r="H41" s="15"/>
       <x:c r="I41" s="15"/>
       <x:c r="J41" s="15"/>
+      <x:c r="K41" s="64"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="18"/>
@@ -1030,10 +1154,11 @@
       <x:c r="D42" s="15"/>
       <x:c r="E42" s="15"/>
       <x:c r="F42" s="21"/>
-      <x:c r="G42" s="15"/>
+      <x:c r="G42" s="18"/>
       <x:c r="H42" s="15"/>
       <x:c r="I42" s="15"/>
       <x:c r="J42" s="15"/>
+      <x:c r="K42" s="64"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="18"/>
@@ -1042,10 +1167,11 @@
       <x:c r="D43" s="15"/>
       <x:c r="E43" s="15"/>
       <x:c r="F43" s="21"/>
-      <x:c r="G43" s="15"/>
+      <x:c r="G43" s="18"/>
       <x:c r="H43" s="15"/>
       <x:c r="I43" s="15"/>
       <x:c r="J43" s="15"/>
+      <x:c r="K43" s="64"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="18"/>
@@ -1054,10 +1180,11 @@
       <x:c r="D44" s="15"/>
       <x:c r="E44" s="15"/>
       <x:c r="F44" s="21"/>
-      <x:c r="G44" s="15"/>
+      <x:c r="G44" s="18"/>
       <x:c r="H44" s="15"/>
       <x:c r="I44" s="15"/>
       <x:c r="J44" s="15"/>
+      <x:c r="K44" s="64"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="18"/>
@@ -1066,10 +1193,11 @@
       <x:c r="D45" s="15"/>
       <x:c r="E45" s="15"/>
       <x:c r="F45" s="21"/>
-      <x:c r="G45" s="15"/>
+      <x:c r="G45" s="18"/>
       <x:c r="H45" s="15"/>
       <x:c r="I45" s="15"/>
       <x:c r="J45" s="15"/>
+      <x:c r="K45" s="64"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="18"/>
@@ -1078,10 +1206,11 @@
       <x:c r="D46" s="15"/>
       <x:c r="E46" s="15"/>
       <x:c r="F46" s="21"/>
-      <x:c r="G46" s="15"/>
+      <x:c r="G46" s="18"/>
       <x:c r="H46" s="15"/>
       <x:c r="I46" s="15"/>
       <x:c r="J46" s="15"/>
+      <x:c r="K46" s="64"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="18"/>
@@ -1090,10 +1219,11 @@
       <x:c r="D47" s="15"/>
       <x:c r="E47" s="15"/>
       <x:c r="F47" s="21"/>
-      <x:c r="G47" s="15"/>
+      <x:c r="G47" s="18"/>
       <x:c r="H47" s="15"/>
       <x:c r="I47" s="15"/>
       <x:c r="J47" s="15"/>
+      <x:c r="K47" s="64"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="18"/>
@@ -1102,10 +1232,11 @@
       <x:c r="D48" s="15"/>
       <x:c r="E48" s="15"/>
       <x:c r="F48" s="21"/>
-      <x:c r="G48" s="15"/>
+      <x:c r="G48" s="18"/>
       <x:c r="H48" s="15"/>
       <x:c r="I48" s="15"/>
       <x:c r="J48" s="15"/>
+      <x:c r="K48" s="64"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="18"/>
@@ -1114,10 +1245,11 @@
       <x:c r="D49" s="15"/>
       <x:c r="E49" s="15"/>
       <x:c r="F49" s="21"/>
-      <x:c r="G49" s="15"/>
+      <x:c r="G49" s="18"/>
       <x:c r="H49" s="15"/>
       <x:c r="I49" s="15"/>
       <x:c r="J49" s="15"/>
+      <x:c r="K49" s="64"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="18"/>
@@ -1126,10 +1258,11 @@
       <x:c r="D50" s="15"/>
       <x:c r="E50" s="15"/>
       <x:c r="F50" s="21"/>
-      <x:c r="G50" s="15"/>
+      <x:c r="G50" s="18"/>
       <x:c r="H50" s="15"/>
       <x:c r="I50" s="15"/>
       <x:c r="J50" s="15"/>
+      <x:c r="K50" s="64"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="18"/>
@@ -1138,10 +1271,11 @@
       <x:c r="D51" s="15"/>
       <x:c r="E51" s="15"/>
       <x:c r="F51" s="21"/>
-      <x:c r="G51" s="15"/>
+      <x:c r="G51" s="18"/>
       <x:c r="H51" s="15"/>
       <x:c r="I51" s="15"/>
       <x:c r="J51" s="15"/>
+      <x:c r="K51" s="64"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="18"/>
@@ -1150,10 +1284,11 @@
       <x:c r="D52" s="15"/>
       <x:c r="E52" s="15"/>
       <x:c r="F52" s="21"/>
-      <x:c r="G52" s="15"/>
+      <x:c r="G52" s="18"/>
       <x:c r="H52" s="15"/>
       <x:c r="I52" s="15"/>
       <x:c r="J52" s="15"/>
+      <x:c r="K52" s="64"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="18"/>
@@ -1162,10 +1297,11 @@
       <x:c r="D53" s="15"/>
       <x:c r="E53" s="15"/>
       <x:c r="F53" s="21"/>
-      <x:c r="G53" s="15"/>
+      <x:c r="G53" s="18"/>
       <x:c r="H53" s="15"/>
       <x:c r="I53" s="15"/>
       <x:c r="J53" s="15"/>
+      <x:c r="K53" s="64"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="18"/>
@@ -1174,10 +1310,11 @@
       <x:c r="D54" s="15"/>
       <x:c r="E54" s="15"/>
       <x:c r="F54" s="21"/>
-      <x:c r="G54" s="15"/>
+      <x:c r="G54" s="18"/>
       <x:c r="H54" s="15"/>
       <x:c r="I54" s="15"/>
       <x:c r="J54" s="15"/>
+      <x:c r="K54" s="64"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="18"/>
@@ -1186,10 +1323,11 @@
       <x:c r="D55" s="15"/>
       <x:c r="E55" s="15"/>
       <x:c r="F55" s="21"/>
-      <x:c r="G55" s="15"/>
+      <x:c r="G55" s="18"/>
       <x:c r="H55" s="15"/>
       <x:c r="I55" s="15"/>
       <x:c r="J55" s="15"/>
+      <x:c r="K55" s="64"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="18"/>
@@ -1198,10 +1336,11 @@
       <x:c r="D56" s="15"/>
       <x:c r="E56" s="15"/>
       <x:c r="F56" s="21"/>
-      <x:c r="G56" s="15"/>
+      <x:c r="G56" s="18"/>
       <x:c r="H56" s="15"/>
       <x:c r="I56" s="15"/>
       <x:c r="J56" s="15"/>
+      <x:c r="K56" s="64"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="18"/>
@@ -1210,10 +1349,11 @@
       <x:c r="D57" s="15"/>
       <x:c r="E57" s="15"/>
       <x:c r="F57" s="21"/>
-      <x:c r="G57" s="15"/>
+      <x:c r="G57" s="18"/>
       <x:c r="H57" s="15"/>
       <x:c r="I57" s="15"/>
       <x:c r="J57" s="15"/>
+      <x:c r="K57" s="64"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="18"/>
@@ -1222,10 +1362,11 @@
       <x:c r="D58" s="15"/>
       <x:c r="E58" s="15"/>
       <x:c r="F58" s="21"/>
-      <x:c r="G58" s="15"/>
+      <x:c r="G58" s="18"/>
       <x:c r="H58" s="15"/>
       <x:c r="I58" s="15"/>
       <x:c r="J58" s="15"/>
+      <x:c r="K58" s="64"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="18"/>
@@ -1234,10 +1375,11 @@
       <x:c r="D59" s="15"/>
       <x:c r="E59" s="15"/>
       <x:c r="F59" s="21"/>
-      <x:c r="G59" s="15"/>
+      <x:c r="G59" s="18"/>
       <x:c r="H59" s="15"/>
       <x:c r="I59" s="15"/>
       <x:c r="J59" s="15"/>
+      <x:c r="K59" s="64"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="18"/>
@@ -1246,10 +1388,11 @@
       <x:c r="D60" s="15"/>
       <x:c r="E60" s="15"/>
       <x:c r="F60" s="21"/>
-      <x:c r="G60" s="15"/>
+      <x:c r="G60" s="18"/>
       <x:c r="H60" s="15"/>
       <x:c r="I60" s="15"/>
       <x:c r="J60" s="15"/>
+      <x:c r="K60" s="64"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="18"/>
@@ -1258,10 +1401,11 @@
       <x:c r="D61" s="15"/>
       <x:c r="E61" s="15"/>
       <x:c r="F61" s="21"/>
-      <x:c r="G61" s="15"/>
+      <x:c r="G61" s="18"/>
       <x:c r="H61" s="15"/>
       <x:c r="I61" s="15"/>
       <x:c r="J61" s="15"/>
+      <x:c r="K61" s="64"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="18"/>
@@ -1270,10 +1414,11 @@
       <x:c r="D62" s="15"/>
       <x:c r="E62" s="15"/>
       <x:c r="F62" s="21"/>
-      <x:c r="G62" s="15"/>
+      <x:c r="G62" s="18"/>
       <x:c r="H62" s="15"/>
       <x:c r="I62" s="15"/>
       <x:c r="J62" s="15"/>
+      <x:c r="K62" s="64"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="18"/>
@@ -1282,10 +1427,11 @@
       <x:c r="D63" s="15"/>
       <x:c r="E63" s="15"/>
       <x:c r="F63" s="21"/>
-      <x:c r="G63" s="15"/>
+      <x:c r="G63" s="18"/>
       <x:c r="H63" s="15"/>
       <x:c r="I63" s="15"/>
       <x:c r="J63" s="15"/>
+      <x:c r="K63" s="64"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="18"/>
@@ -1294,10 +1440,11 @@
       <x:c r="D64" s="15"/>
       <x:c r="E64" s="15"/>
       <x:c r="F64" s="21"/>
-      <x:c r="G64" s="15"/>
+      <x:c r="G64" s="18"/>
       <x:c r="H64" s="15"/>
       <x:c r="I64" s="15"/>
       <x:c r="J64" s="15"/>
+      <x:c r="K64" s="64"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="18"/>
@@ -1306,10 +1453,11 @@
       <x:c r="D65" s="15"/>
       <x:c r="E65" s="15"/>
       <x:c r="F65" s="21"/>
-      <x:c r="G65" s="15"/>
+      <x:c r="G65" s="18"/>
       <x:c r="H65" s="15"/>
       <x:c r="I65" s="15"/>
       <x:c r="J65" s="15"/>
+      <x:c r="K65" s="64"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="18"/>
@@ -1318,10 +1466,11 @@
       <x:c r="D66" s="15"/>
       <x:c r="E66" s="15"/>
       <x:c r="F66" s="21"/>
-      <x:c r="G66" s="15"/>
+      <x:c r="G66" s="18"/>
       <x:c r="H66" s="15"/>
       <x:c r="I66" s="15"/>
       <x:c r="J66" s="15"/>
+      <x:c r="K66" s="64"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="18"/>
@@ -1330,10 +1479,11 @@
       <x:c r="D67" s="15"/>
       <x:c r="E67" s="15"/>
       <x:c r="F67" s="21"/>
-      <x:c r="G67" s="15"/>
+      <x:c r="G67" s="18"/>
       <x:c r="H67" s="15"/>
       <x:c r="I67" s="15"/>
       <x:c r="J67" s="15"/>
+      <x:c r="K67" s="64"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="18"/>
@@ -1342,10 +1492,11 @@
       <x:c r="D68" s="15"/>
       <x:c r="E68" s="15"/>
       <x:c r="F68" s="21"/>
-      <x:c r="G68" s="15"/>
+      <x:c r="G68" s="18"/>
       <x:c r="H68" s="15"/>
       <x:c r="I68" s="15"/>
       <x:c r="J68" s="15"/>
+      <x:c r="K68" s="64"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="18"/>
@@ -1354,10 +1505,11 @@
       <x:c r="D69" s="15"/>
       <x:c r="E69" s="15"/>
       <x:c r="F69" s="21"/>
-      <x:c r="G69" s="15"/>
+      <x:c r="G69" s="18"/>
       <x:c r="H69" s="15"/>
       <x:c r="I69" s="15"/>
       <x:c r="J69" s="15"/>
+      <x:c r="K69" s="64"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="18"/>
@@ -1366,10 +1518,11 @@
       <x:c r="D70" s="15"/>
       <x:c r="E70" s="15"/>
       <x:c r="F70" s="21"/>
-      <x:c r="G70" s="15"/>
+      <x:c r="G70" s="18"/>
       <x:c r="H70" s="15"/>
       <x:c r="I70" s="15"/>
       <x:c r="J70" s="15"/>
+      <x:c r="K70" s="64"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="18"/>
@@ -1378,10 +1531,11 @@
       <x:c r="D71" s="15"/>
       <x:c r="E71" s="15"/>
       <x:c r="F71" s="21"/>
-      <x:c r="G71" s="15"/>
+      <x:c r="G71" s="18"/>
       <x:c r="H71" s="15"/>
       <x:c r="I71" s="15"/>
       <x:c r="J71" s="15"/>
+      <x:c r="K71" s="64"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="18"/>
@@ -1390,10 +1544,11 @@
       <x:c r="D72" s="15"/>
       <x:c r="E72" s="15"/>
       <x:c r="F72" s="21"/>
-      <x:c r="G72" s="15"/>
+      <x:c r="G72" s="18"/>
       <x:c r="H72" s="15"/>
       <x:c r="I72" s="15"/>
       <x:c r="J72" s="15"/>
+      <x:c r="K72" s="64"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="18"/>
@@ -1402,10 +1557,11 @@
       <x:c r="D73" s="15"/>
       <x:c r="E73" s="15"/>
       <x:c r="F73" s="21"/>
-      <x:c r="G73" s="15"/>
+      <x:c r="G73" s="18"/>
       <x:c r="H73" s="15"/>
       <x:c r="I73" s="15"/>
       <x:c r="J73" s="15"/>
+      <x:c r="K73" s="64"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="18"/>
@@ -1414,10 +1570,11 @@
       <x:c r="D74" s="15"/>
       <x:c r="E74" s="15"/>
       <x:c r="F74" s="21"/>
-      <x:c r="G74" s="15"/>
+      <x:c r="G74" s="18"/>
       <x:c r="H74" s="15"/>
       <x:c r="I74" s="15"/>
       <x:c r="J74" s="15"/>
+      <x:c r="K74" s="64"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="18"/>
@@ -1426,10 +1583,11 @@
       <x:c r="D75" s="15"/>
       <x:c r="E75" s="15"/>
       <x:c r="F75" s="21"/>
-      <x:c r="G75" s="15"/>
+      <x:c r="G75" s="18"/>
       <x:c r="H75" s="15"/>
       <x:c r="I75" s="15"/>
       <x:c r="J75" s="15"/>
+      <x:c r="K75" s="64"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="18"/>
@@ -1438,10 +1596,11 @@
       <x:c r="D76" s="15"/>
       <x:c r="E76" s="15"/>
       <x:c r="F76" s="21"/>
-      <x:c r="G76" s="15"/>
+      <x:c r="G76" s="18"/>
       <x:c r="H76" s="15"/>
       <x:c r="I76" s="15"/>
       <x:c r="J76" s="15"/>
+      <x:c r="K76" s="64"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="18"/>
@@ -1450,10 +1609,11 @@
       <x:c r="D77" s="15"/>
       <x:c r="E77" s="15"/>
       <x:c r="F77" s="21"/>
-      <x:c r="G77" s="15"/>
+      <x:c r="G77" s="18"/>
       <x:c r="H77" s="15"/>
       <x:c r="I77" s="15"/>
       <x:c r="J77" s="15"/>
+      <x:c r="K77" s="64"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="18"/>
@@ -1462,10 +1622,11 @@
       <x:c r="D78" s="15"/>
       <x:c r="E78" s="15"/>
       <x:c r="F78" s="21"/>
-      <x:c r="G78" s="15"/>
+      <x:c r="G78" s="18"/>
       <x:c r="H78" s="15"/>
       <x:c r="I78" s="15"/>
       <x:c r="J78" s="15"/>
+      <x:c r="K78" s="64"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="18"/>
@@ -1474,10 +1635,11 @@
       <x:c r="D79" s="15"/>
       <x:c r="E79" s="15"/>
       <x:c r="F79" s="21"/>
-      <x:c r="G79" s="15"/>
+      <x:c r="G79" s="18"/>
       <x:c r="H79" s="15"/>
       <x:c r="I79" s="15"/>
       <x:c r="J79" s="15"/>
+      <x:c r="K79" s="64"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="18"/>
@@ -1486,10 +1648,11 @@
       <x:c r="D80" s="15"/>
       <x:c r="E80" s="15"/>
       <x:c r="F80" s="21"/>
-      <x:c r="G80" s="15"/>
+      <x:c r="G80" s="18"/>
       <x:c r="H80" s="15"/>
       <x:c r="I80" s="15"/>
       <x:c r="J80" s="15"/>
+      <x:c r="K80" s="64"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="18"/>
@@ -1498,10 +1661,11 @@
       <x:c r="D81" s="15"/>
       <x:c r="E81" s="15"/>
       <x:c r="F81" s="21"/>
-      <x:c r="G81" s="15"/>
+      <x:c r="G81" s="18"/>
       <x:c r="H81" s="15"/>
       <x:c r="I81" s="15"/>
       <x:c r="J81" s="15"/>
+      <x:c r="K81" s="64"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="18"/>
@@ -1510,10 +1674,11 @@
       <x:c r="D82" s="15"/>
       <x:c r="E82" s="15"/>
       <x:c r="F82" s="21"/>
-      <x:c r="G82" s="15"/>
+      <x:c r="G82" s="18"/>
       <x:c r="H82" s="15"/>
       <x:c r="I82" s="15"/>
       <x:c r="J82" s="15"/>
+      <x:c r="K82" s="64"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="18"/>
@@ -1522,10 +1687,11 @@
       <x:c r="D83" s="15"/>
       <x:c r="E83" s="15"/>
       <x:c r="F83" s="21"/>
-      <x:c r="G83" s="15"/>
+      <x:c r="G83" s="18"/>
       <x:c r="H83" s="15"/>
       <x:c r="I83" s="15"/>
       <x:c r="J83" s="15"/>
+      <x:c r="K83" s="64"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="18"/>
@@ -1534,10 +1700,11 @@
       <x:c r="D84" s="15"/>
       <x:c r="E84" s="15"/>
       <x:c r="F84" s="21"/>
-      <x:c r="G84" s="15"/>
+      <x:c r="G84" s="18"/>
       <x:c r="H84" s="15"/>
       <x:c r="I84" s="15"/>
       <x:c r="J84" s="15"/>
+      <x:c r="K84" s="64"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="18"/>
@@ -1546,10 +1713,11 @@
       <x:c r="D85" s="15"/>
       <x:c r="E85" s="15"/>
       <x:c r="F85" s="21"/>
-      <x:c r="G85" s="15"/>
+      <x:c r="G85" s="18"/>
       <x:c r="H85" s="15"/>
       <x:c r="I85" s="15"/>
       <x:c r="J85" s="15"/>
+      <x:c r="K85" s="64"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="18"/>
@@ -1558,10 +1726,11 @@
       <x:c r="D86" s="15"/>
       <x:c r="E86" s="15"/>
       <x:c r="F86" s="21"/>
-      <x:c r="G86" s="15"/>
+      <x:c r="G86" s="18"/>
       <x:c r="H86" s="15"/>
       <x:c r="I86" s="15"/>
       <x:c r="J86" s="15"/>
+      <x:c r="K86" s="64"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="18"/>
@@ -1570,10 +1739,11 @@
       <x:c r="D87" s="15"/>
       <x:c r="E87" s="15"/>
       <x:c r="F87" s="21"/>
-      <x:c r="G87" s="15"/>
+      <x:c r="G87" s="18"/>
       <x:c r="H87" s="15"/>
       <x:c r="I87" s="15"/>
       <x:c r="J87" s="15"/>
+      <x:c r="K87" s="64"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="18"/>
@@ -1582,10 +1752,11 @@
       <x:c r="D88" s="15"/>
       <x:c r="E88" s="15"/>
       <x:c r="F88" s="21"/>
-      <x:c r="G88" s="15"/>
+      <x:c r="G88" s="18"/>
       <x:c r="H88" s="15"/>
       <x:c r="I88" s="15"/>
       <x:c r="J88" s="15"/>
+      <x:c r="K88" s="64"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="18"/>
@@ -1594,10 +1765,11 @@
       <x:c r="D89" s="15"/>
       <x:c r="E89" s="15"/>
       <x:c r="F89" s="21"/>
-      <x:c r="G89" s="15"/>
+      <x:c r="G89" s="18"/>
       <x:c r="H89" s="15"/>
       <x:c r="I89" s="15"/>
       <x:c r="J89" s="15"/>
+      <x:c r="K89" s="64"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="18"/>
@@ -1606,10 +1778,11 @@
       <x:c r="D90" s="15"/>
       <x:c r="E90" s="15"/>
       <x:c r="F90" s="21"/>
-      <x:c r="G90" s="15"/>
+      <x:c r="G90" s="18"/>
       <x:c r="H90" s="15"/>
       <x:c r="I90" s="15"/>
       <x:c r="J90" s="15"/>
+      <x:c r="K90" s="64"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="18"/>
@@ -1618,10 +1791,11 @@
       <x:c r="D91" s="15"/>
       <x:c r="E91" s="15"/>
       <x:c r="F91" s="21"/>
-      <x:c r="G91" s="15"/>
+      <x:c r="G91" s="18"/>
       <x:c r="H91" s="15"/>
       <x:c r="I91" s="15"/>
       <x:c r="J91" s="15"/>
+      <x:c r="K91" s="64"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="18"/>
@@ -1630,10 +1804,11 @@
       <x:c r="D92" s="15"/>
       <x:c r="E92" s="15"/>
       <x:c r="F92" s="21"/>
-      <x:c r="G92" s="15"/>
+      <x:c r="G92" s="18"/>
       <x:c r="H92" s="15"/>
       <x:c r="I92" s="15"/>
       <x:c r="J92" s="15"/>
+      <x:c r="K92" s="64"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="18"/>
@@ -1642,10 +1817,11 @@
       <x:c r="D93" s="15"/>
       <x:c r="E93" s="15"/>
       <x:c r="F93" s="21"/>
-      <x:c r="G93" s="15"/>
+      <x:c r="G93" s="18"/>
       <x:c r="H93" s="15"/>
       <x:c r="I93" s="15"/>
       <x:c r="J93" s="15"/>
+      <x:c r="K93" s="64"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="18"/>
@@ -1654,10 +1830,11 @@
       <x:c r="D94" s="15"/>
       <x:c r="E94" s="15"/>
       <x:c r="F94" s="21"/>
-      <x:c r="G94" s="15"/>
+      <x:c r="G94" s="18"/>
       <x:c r="H94" s="15"/>
       <x:c r="I94" s="15"/>
       <x:c r="J94" s="15"/>
+      <x:c r="K94" s="64"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="18"/>
@@ -1666,10 +1843,11 @@
       <x:c r="D95" s="15"/>
       <x:c r="E95" s="15"/>
       <x:c r="F95" s="21"/>
-      <x:c r="G95" s="15"/>
+      <x:c r="G95" s="18"/>
       <x:c r="H95" s="15"/>
       <x:c r="I95" s="15"/>
       <x:c r="J95" s="15"/>
+      <x:c r="K95" s="64"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="18"/>
@@ -1678,10 +1856,11 @@
       <x:c r="D96" s="15"/>
       <x:c r="E96" s="15"/>
       <x:c r="F96" s="21"/>
-      <x:c r="G96" s="15"/>
+      <x:c r="G96" s="18"/>
       <x:c r="H96" s="15"/>
       <x:c r="I96" s="15"/>
       <x:c r="J96" s="15"/>
+      <x:c r="K96" s="64"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="18"/>
@@ -1690,10 +1869,11 @@
       <x:c r="D97" s="15"/>
       <x:c r="E97" s="15"/>
       <x:c r="F97" s="21"/>
-      <x:c r="G97" s="15"/>
+      <x:c r="G97" s="18"/>
       <x:c r="H97" s="15"/>
       <x:c r="I97" s="15"/>
       <x:c r="J97" s="15"/>
+      <x:c r="K97" s="64"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="18"/>
@@ -1702,10 +1882,11 @@
       <x:c r="D98" s="15"/>
       <x:c r="E98" s="15"/>
       <x:c r="F98" s="21"/>
-      <x:c r="G98" s="15"/>
+      <x:c r="G98" s="18"/>
       <x:c r="H98" s="15"/>
       <x:c r="I98" s="15"/>
       <x:c r="J98" s="15"/>
+      <x:c r="K98" s="64"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="18"/>
@@ -1714,10 +1895,11 @@
       <x:c r="D99" s="15"/>
       <x:c r="E99" s="15"/>
       <x:c r="F99" s="21"/>
-      <x:c r="G99" s="15"/>
+      <x:c r="G99" s="18"/>
       <x:c r="H99" s="15"/>
       <x:c r="I99" s="15"/>
       <x:c r="J99" s="15"/>
+      <x:c r="K99" s="64"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="18"/>
@@ -1726,10 +1908,11 @@
       <x:c r="D100" s="15"/>
       <x:c r="E100" s="15"/>
       <x:c r="F100" s="21"/>
-      <x:c r="G100" s="15"/>
+      <x:c r="G100" s="18"/>
       <x:c r="H100" s="15"/>
       <x:c r="I100" s="15"/>
       <x:c r="J100" s="15"/>
+      <x:c r="K100" s="64"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="19"/>
@@ -1738,15 +1921,2819 @@
       <x:c r="D101" s="16"/>
       <x:c r="E101" s="16"/>
       <x:c r="F101" s="22"/>
-      <x:c r="G101" s="16"/>
+      <x:c r="G101" s="19"/>
       <x:c r="H101" s="16"/>
       <x:c r="I101" s="16"/>
       <x:c r="J101" s="16"/>
+      <x:c r="K101" s="64"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="G102" s="57"/>
+      <x:c r="H102"/>
+      <x:c r="I102"/>
+      <x:c r="J102"/>
+      <x:c r="K102" s="64"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="G103" s="57"/>
+      <x:c r="H103"/>
+      <x:c r="I103"/>
+      <x:c r="J103"/>
+      <x:c r="K103" s="64"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="G104" s="57"/>
+      <x:c r="H104"/>
+      <x:c r="I104"/>
+      <x:c r="J104"/>
+      <x:c r="K104" s="64"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="G105" s="57"/>
+      <x:c r="H105"/>
+      <x:c r="I105"/>
+      <x:c r="J105"/>
+      <x:c r="K105" s="64"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="G106" s="57"/>
+      <x:c r="H106"/>
+      <x:c r="I106"/>
+      <x:c r="J106"/>
+      <x:c r="K106" s="64"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="G107" s="57"/>
+      <x:c r="H107"/>
+      <x:c r="I107"/>
+      <x:c r="J107"/>
+      <x:c r="K107" s="64"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="G108" s="57"/>
+      <x:c r="H108"/>
+      <x:c r="I108"/>
+      <x:c r="J108"/>
+      <x:c r="K108" s="64"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="G109" s="57"/>
+      <x:c r="H109"/>
+      <x:c r="I109"/>
+      <x:c r="J109"/>
+      <x:c r="K109" s="64"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="G110" s="57"/>
+      <x:c r="H110"/>
+      <x:c r="I110"/>
+      <x:c r="J110"/>
+      <x:c r="K110" s="64"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="G111" s="57"/>
+      <x:c r="H111"/>
+      <x:c r="I111"/>
+      <x:c r="J111"/>
+      <x:c r="K111" s="64"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="G112" s="57"/>
+      <x:c r="H112"/>
+      <x:c r="I112"/>
+      <x:c r="J112"/>
+      <x:c r="K112" s="64"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="G113" s="57"/>
+      <x:c r="H113"/>
+      <x:c r="I113"/>
+      <x:c r="J113"/>
+      <x:c r="K113" s="64"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="G114" s="57"/>
+      <x:c r="H114"/>
+      <x:c r="I114"/>
+      <x:c r="J114"/>
+      <x:c r="K114" s="64"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="G115" s="57"/>
+      <x:c r="H115"/>
+      <x:c r="I115"/>
+      <x:c r="J115"/>
+      <x:c r="K115" s="64"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="G116" s="57"/>
+      <x:c r="H116"/>
+      <x:c r="I116"/>
+      <x:c r="J116"/>
+      <x:c r="K116" s="64"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="G117" s="57"/>
+      <x:c r="H117"/>
+      <x:c r="I117"/>
+      <x:c r="J117"/>
+      <x:c r="K117" s="64"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="G118" s="57"/>
+      <x:c r="H118"/>
+      <x:c r="I118"/>
+      <x:c r="J118"/>
+      <x:c r="K118" s="64"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="G119" s="57"/>
+      <x:c r="H119"/>
+      <x:c r="I119"/>
+      <x:c r="J119"/>
+      <x:c r="K119" s="64"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="G120" s="57"/>
+      <x:c r="H120"/>
+      <x:c r="I120"/>
+      <x:c r="J120"/>
+      <x:c r="K120" s="64"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="G121" s="57"/>
+      <x:c r="H121"/>
+      <x:c r="I121"/>
+      <x:c r="J121"/>
+      <x:c r="K121" s="64"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="G122" s="57"/>
+      <x:c r="H122"/>
+      <x:c r="I122"/>
+      <x:c r="J122"/>
+      <x:c r="K122" s="64"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="G123" s="57"/>
+      <x:c r="H123"/>
+      <x:c r="I123"/>
+      <x:c r="J123"/>
+      <x:c r="K123" s="64"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="G124" s="57"/>
+      <x:c r="H124"/>
+      <x:c r="I124"/>
+      <x:c r="J124"/>
+      <x:c r="K124" s="64"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="G125" s="57"/>
+      <x:c r="H125"/>
+      <x:c r="I125"/>
+      <x:c r="J125"/>
+      <x:c r="K125" s="64"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="G126" s="57"/>
+      <x:c r="H126"/>
+      <x:c r="I126"/>
+      <x:c r="J126"/>
+      <x:c r="K126" s="64"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="G127" s="57"/>
+      <x:c r="H127"/>
+      <x:c r="I127"/>
+      <x:c r="J127"/>
+      <x:c r="K127" s="64"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="G128" s="57"/>
+      <x:c r="H128"/>
+      <x:c r="I128"/>
+      <x:c r="J128"/>
+      <x:c r="K128" s="64"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="G129" s="57"/>
+      <x:c r="H129"/>
+      <x:c r="I129"/>
+      <x:c r="J129"/>
+      <x:c r="K129" s="64"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="G130" s="57"/>
+      <x:c r="H130"/>
+      <x:c r="I130"/>
+      <x:c r="J130"/>
+      <x:c r="K130" s="64"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="G131" s="57"/>
+      <x:c r="H131"/>
+      <x:c r="I131"/>
+      <x:c r="J131"/>
+      <x:c r="K131" s="64"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="G132" s="57"/>
+      <x:c r="H132"/>
+      <x:c r="I132"/>
+      <x:c r="J132"/>
+      <x:c r="K132" s="64"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="G133" s="57"/>
+      <x:c r="H133"/>
+      <x:c r="I133"/>
+      <x:c r="J133"/>
+      <x:c r="K133" s="64"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="G134" s="57"/>
+      <x:c r="H134"/>
+      <x:c r="I134"/>
+      <x:c r="J134"/>
+      <x:c r="K134" s="64"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="G135" s="57"/>
+      <x:c r="H135"/>
+      <x:c r="I135"/>
+      <x:c r="J135"/>
+      <x:c r="K135" s="64"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="G136" s="57"/>
+      <x:c r="H136"/>
+      <x:c r="I136"/>
+      <x:c r="J136"/>
+      <x:c r="K136" s="64"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="G137" s="57"/>
+      <x:c r="H137"/>
+      <x:c r="I137"/>
+      <x:c r="J137"/>
+      <x:c r="K137" s="64"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="G138" s="57"/>
+      <x:c r="H138"/>
+      <x:c r="I138"/>
+      <x:c r="J138"/>
+      <x:c r="K138" s="64"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="G139" s="57"/>
+      <x:c r="H139"/>
+      <x:c r="I139"/>
+      <x:c r="J139"/>
+      <x:c r="K139" s="64"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="G140" s="57"/>
+      <x:c r="H140"/>
+      <x:c r="I140"/>
+      <x:c r="J140"/>
+      <x:c r="K140" s="64"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="G141" s="57"/>
+      <x:c r="H141"/>
+      <x:c r="I141"/>
+      <x:c r="J141"/>
+      <x:c r="K141" s="64"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="G142" s="57"/>
+      <x:c r="H142"/>
+      <x:c r="I142"/>
+      <x:c r="J142"/>
+      <x:c r="K142" s="64"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="G143" s="57"/>
+      <x:c r="H143"/>
+      <x:c r="I143"/>
+      <x:c r="J143"/>
+      <x:c r="K143" s="64"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="G144" s="57"/>
+      <x:c r="H144"/>
+      <x:c r="I144"/>
+      <x:c r="J144"/>
+      <x:c r="K144" s="64"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="G145" s="57"/>
+      <x:c r="H145"/>
+      <x:c r="I145"/>
+      <x:c r="J145"/>
+      <x:c r="K145" s="64"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="G146" s="57"/>
+      <x:c r="H146"/>
+      <x:c r="I146"/>
+      <x:c r="J146"/>
+      <x:c r="K146" s="64"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="G147" s="57"/>
+      <x:c r="H147"/>
+      <x:c r="I147"/>
+      <x:c r="J147"/>
+      <x:c r="K147" s="64"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="G148" s="57"/>
+      <x:c r="H148"/>
+      <x:c r="I148"/>
+      <x:c r="J148"/>
+      <x:c r="K148" s="64"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="G149" s="57"/>
+      <x:c r="H149"/>
+      <x:c r="I149"/>
+      <x:c r="J149"/>
+      <x:c r="K149" s="64"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="G150" s="57"/>
+      <x:c r="H150"/>
+      <x:c r="I150"/>
+      <x:c r="J150"/>
+      <x:c r="K150" s="64"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="G151" s="57"/>
+      <x:c r="H151"/>
+      <x:c r="I151"/>
+      <x:c r="J151"/>
+      <x:c r="K151" s="64"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="G152" s="57"/>
+      <x:c r="H152"/>
+      <x:c r="I152"/>
+      <x:c r="J152"/>
+      <x:c r="K152" s="64"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="G153" s="57"/>
+      <x:c r="H153"/>
+      <x:c r="I153"/>
+      <x:c r="J153"/>
+      <x:c r="K153" s="64"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="G154" s="57"/>
+      <x:c r="H154"/>
+      <x:c r="I154"/>
+      <x:c r="J154"/>
+      <x:c r="K154" s="64"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="G155" s="57"/>
+      <x:c r="H155"/>
+      <x:c r="I155"/>
+      <x:c r="J155"/>
+      <x:c r="K155" s="64"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="G156" s="57"/>
+      <x:c r="H156"/>
+      <x:c r="I156"/>
+      <x:c r="J156"/>
+      <x:c r="K156" s="64"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="G157" s="57"/>
+      <x:c r="H157"/>
+      <x:c r="I157"/>
+      <x:c r="J157"/>
+      <x:c r="K157" s="64"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="G158" s="57"/>
+      <x:c r="H158"/>
+      <x:c r="I158"/>
+      <x:c r="J158"/>
+      <x:c r="K158" s="64"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="G159" s="57"/>
+      <x:c r="H159"/>
+      <x:c r="I159"/>
+      <x:c r="J159"/>
+      <x:c r="K159" s="64"/>
+    </x:row>
+    <x:row r="160">
+      <x:c r="G160" s="57"/>
+      <x:c r="H160"/>
+      <x:c r="I160"/>
+      <x:c r="J160"/>
+      <x:c r="K160" s="64"/>
+    </x:row>
+    <x:row r="161">
+      <x:c r="G161" s="57"/>
+      <x:c r="H161"/>
+      <x:c r="I161"/>
+      <x:c r="J161"/>
+      <x:c r="K161" s="64"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="G162" s="57"/>
+      <x:c r="H162"/>
+      <x:c r="I162"/>
+      <x:c r="J162"/>
+      <x:c r="K162" s="64"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="G163" s="57"/>
+      <x:c r="H163"/>
+      <x:c r="I163"/>
+      <x:c r="J163"/>
+      <x:c r="K163" s="64"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="G164" s="57"/>
+      <x:c r="H164"/>
+      <x:c r="I164"/>
+      <x:c r="J164"/>
+      <x:c r="K164" s="64"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="G165" s="57"/>
+      <x:c r="H165"/>
+      <x:c r="I165"/>
+      <x:c r="J165"/>
+      <x:c r="K165" s="64"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="G166" s="57"/>
+      <x:c r="H166"/>
+      <x:c r="I166"/>
+      <x:c r="J166"/>
+      <x:c r="K166" s="64"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="G167" s="57"/>
+      <x:c r="H167"/>
+      <x:c r="I167"/>
+      <x:c r="J167"/>
+      <x:c r="K167" s="64"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="G168" s="57"/>
+      <x:c r="H168"/>
+      <x:c r="I168"/>
+      <x:c r="J168"/>
+      <x:c r="K168" s="64"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="G169" s="57"/>
+      <x:c r="H169"/>
+      <x:c r="I169"/>
+      <x:c r="J169"/>
+      <x:c r="K169" s="64"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="G170" s="57"/>
+      <x:c r="H170"/>
+      <x:c r="I170"/>
+      <x:c r="J170"/>
+      <x:c r="K170" s="64"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="G171" s="57"/>
+      <x:c r="H171"/>
+      <x:c r="I171"/>
+      <x:c r="J171"/>
+      <x:c r="K171" s="64"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="G172" s="57"/>
+      <x:c r="H172"/>
+      <x:c r="I172"/>
+      <x:c r="J172"/>
+      <x:c r="K172" s="64"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="G173" s="57"/>
+      <x:c r="H173"/>
+      <x:c r="I173"/>
+      <x:c r="J173"/>
+      <x:c r="K173" s="64"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="G174" s="57"/>
+      <x:c r="H174"/>
+      <x:c r="I174"/>
+      <x:c r="J174"/>
+      <x:c r="K174" s="64"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="G175" s="57"/>
+      <x:c r="H175"/>
+      <x:c r="I175"/>
+      <x:c r="J175"/>
+      <x:c r="K175" s="64"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="G176" s="57"/>
+      <x:c r="H176"/>
+      <x:c r="I176"/>
+      <x:c r="J176"/>
+      <x:c r="K176" s="64"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="G177" s="57"/>
+      <x:c r="H177"/>
+      <x:c r="I177"/>
+      <x:c r="J177"/>
+      <x:c r="K177" s="64"/>
+    </x:row>
+    <x:row r="178">
+      <x:c r="G178" s="57"/>
+      <x:c r="H178"/>
+      <x:c r="I178"/>
+      <x:c r="J178"/>
+      <x:c r="K178" s="64"/>
+    </x:row>
+    <x:row r="179">
+      <x:c r="G179" s="57"/>
+      <x:c r="H179"/>
+      <x:c r="I179"/>
+      <x:c r="J179"/>
+      <x:c r="K179" s="64"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="G180" s="57"/>
+      <x:c r="H180"/>
+      <x:c r="I180"/>
+      <x:c r="J180"/>
+      <x:c r="K180" s="64"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="G181" s="57"/>
+      <x:c r="H181"/>
+      <x:c r="I181"/>
+      <x:c r="J181"/>
+      <x:c r="K181" s="64"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="G182" s="57"/>
+      <x:c r="H182"/>
+      <x:c r="I182"/>
+      <x:c r="J182"/>
+      <x:c r="K182" s="64"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="G183" s="57"/>
+      <x:c r="H183"/>
+      <x:c r="I183"/>
+      <x:c r="J183"/>
+      <x:c r="K183" s="64"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="G184" s="57"/>
+      <x:c r="H184"/>
+      <x:c r="I184"/>
+      <x:c r="J184"/>
+      <x:c r="K184" s="64"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="G185" s="57"/>
+      <x:c r="H185"/>
+      <x:c r="I185"/>
+      <x:c r="J185"/>
+      <x:c r="K185" s="64"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="G186" s="57"/>
+      <x:c r="H186"/>
+      <x:c r="I186"/>
+      <x:c r="J186"/>
+      <x:c r="K186" s="64"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="G187" s="57"/>
+      <x:c r="H187"/>
+      <x:c r="I187"/>
+      <x:c r="J187"/>
+      <x:c r="K187" s="64"/>
+    </x:row>
+    <x:row r="188">
+      <x:c r="G188" s="57"/>
+      <x:c r="H188"/>
+      <x:c r="I188"/>
+      <x:c r="J188"/>
+      <x:c r="K188" s="64"/>
+    </x:row>
+    <x:row r="189">
+      <x:c r="G189" s="57"/>
+      <x:c r="H189"/>
+      <x:c r="I189"/>
+      <x:c r="J189"/>
+      <x:c r="K189" s="64"/>
+    </x:row>
+    <x:row r="190">
+      <x:c r="G190" s="57"/>
+      <x:c r="H190"/>
+      <x:c r="I190"/>
+      <x:c r="J190"/>
+      <x:c r="K190" s="64"/>
+    </x:row>
+    <x:row r="191">
+      <x:c r="G191" s="57"/>
+      <x:c r="H191"/>
+      <x:c r="I191"/>
+      <x:c r="J191"/>
+      <x:c r="K191" s="64"/>
+    </x:row>
+    <x:row r="192">
+      <x:c r="G192" s="57"/>
+      <x:c r="H192"/>
+      <x:c r="I192"/>
+      <x:c r="J192"/>
+      <x:c r="K192" s="64"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="G193" s="57"/>
+      <x:c r="H193"/>
+      <x:c r="I193"/>
+      <x:c r="J193"/>
+      <x:c r="K193" s="64"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="G194" s="57"/>
+      <x:c r="H194"/>
+      <x:c r="I194"/>
+      <x:c r="J194"/>
+      <x:c r="K194" s="64"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="G195" s="57"/>
+      <x:c r="H195"/>
+      <x:c r="I195"/>
+      <x:c r="J195"/>
+      <x:c r="K195" s="64"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="G196" s="57"/>
+      <x:c r="H196"/>
+      <x:c r="I196"/>
+      <x:c r="J196"/>
+      <x:c r="K196" s="64"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="G197" s="57"/>
+      <x:c r="H197"/>
+      <x:c r="I197"/>
+      <x:c r="J197"/>
+      <x:c r="K197" s="64"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="G198" s="57"/>
+      <x:c r="H198"/>
+      <x:c r="I198"/>
+      <x:c r="J198"/>
+      <x:c r="K198" s="64"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="G199" s="57"/>
+      <x:c r="H199"/>
+      <x:c r="I199"/>
+      <x:c r="J199"/>
+      <x:c r="K199" s="64"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="G200" s="57"/>
+      <x:c r="H200"/>
+      <x:c r="I200"/>
+      <x:c r="J200"/>
+      <x:c r="K200" s="64"/>
+    </x:row>
+    <x:row r="201">
+      <x:c r="G201" s="57"/>
+      <x:c r="H201"/>
+      <x:c r="I201"/>
+      <x:c r="J201"/>
+      <x:c r="K201" s="64"/>
+    </x:row>
+    <x:row r="202">
+      <x:c r="G202" s="57"/>
+      <x:c r="H202"/>
+      <x:c r="I202"/>
+      <x:c r="J202"/>
+      <x:c r="K202" s="64"/>
+    </x:row>
+    <x:row r="203">
+      <x:c r="G203" s="57"/>
+      <x:c r="H203"/>
+      <x:c r="I203"/>
+      <x:c r="J203"/>
+      <x:c r="K203" s="64"/>
+    </x:row>
+    <x:row r="204">
+      <x:c r="G204" s="57"/>
+      <x:c r="H204"/>
+      <x:c r="I204"/>
+      <x:c r="J204"/>
+      <x:c r="K204" s="64"/>
+    </x:row>
+    <x:row r="205">
+      <x:c r="G205" s="57"/>
+      <x:c r="H205"/>
+      <x:c r="I205"/>
+      <x:c r="J205"/>
+      <x:c r="K205" s="64"/>
+    </x:row>
+    <x:row r="206">
+      <x:c r="G206" s="57"/>
+      <x:c r="H206"/>
+      <x:c r="I206"/>
+      <x:c r="J206"/>
+      <x:c r="K206" s="64"/>
+    </x:row>
+    <x:row r="207">
+      <x:c r="G207" s="57"/>
+      <x:c r="H207"/>
+      <x:c r="I207"/>
+      <x:c r="J207"/>
+      <x:c r="K207" s="64"/>
+    </x:row>
+    <x:row r="208">
+      <x:c r="G208" s="57"/>
+      <x:c r="H208"/>
+      <x:c r="I208"/>
+      <x:c r="J208"/>
+      <x:c r="K208" s="64"/>
+    </x:row>
+    <x:row r="209">
+      <x:c r="G209" s="57"/>
+      <x:c r="H209"/>
+      <x:c r="I209"/>
+      <x:c r="J209"/>
+      <x:c r="K209" s="64"/>
+    </x:row>
+    <x:row r="210">
+      <x:c r="G210" s="57"/>
+      <x:c r="H210"/>
+      <x:c r="I210"/>
+      <x:c r="J210"/>
+      <x:c r="K210" s="64"/>
+    </x:row>
+    <x:row r="211">
+      <x:c r="G211" s="57"/>
+      <x:c r="H211"/>
+      <x:c r="I211"/>
+      <x:c r="J211"/>
+      <x:c r="K211" s="64"/>
+    </x:row>
+    <x:row r="212">
+      <x:c r="G212" s="57"/>
+      <x:c r="H212"/>
+      <x:c r="I212"/>
+      <x:c r="J212"/>
+      <x:c r="K212" s="64"/>
+    </x:row>
+    <x:row r="213">
+      <x:c r="G213" s="57"/>
+      <x:c r="H213"/>
+      <x:c r="I213"/>
+      <x:c r="J213"/>
+      <x:c r="K213" s="64"/>
+    </x:row>
+    <x:row r="214">
+      <x:c r="G214" s="57"/>
+      <x:c r="H214"/>
+      <x:c r="I214"/>
+      <x:c r="J214"/>
+      <x:c r="K214" s="64"/>
+    </x:row>
+    <x:row r="215">
+      <x:c r="G215" s="57"/>
+      <x:c r="H215"/>
+      <x:c r="I215"/>
+      <x:c r="J215"/>
+      <x:c r="K215" s="64"/>
+    </x:row>
+    <x:row r="216">
+      <x:c r="G216" s="57"/>
+      <x:c r="H216"/>
+      <x:c r="I216"/>
+      <x:c r="J216"/>
+      <x:c r="K216" s="64"/>
+    </x:row>
+    <x:row r="217">
+      <x:c r="G217" s="57"/>
+      <x:c r="H217"/>
+      <x:c r="I217"/>
+      <x:c r="J217"/>
+      <x:c r="K217" s="64"/>
+    </x:row>
+    <x:row r="218">
+      <x:c r="G218" s="57"/>
+      <x:c r="H218"/>
+      <x:c r="I218"/>
+      <x:c r="J218"/>
+      <x:c r="K218" s="64"/>
+    </x:row>
+    <x:row r="219">
+      <x:c r="G219" s="57"/>
+      <x:c r="H219"/>
+      <x:c r="I219"/>
+      <x:c r="J219"/>
+      <x:c r="K219" s="64"/>
+    </x:row>
+    <x:row r="220">
+      <x:c r="G220" s="57"/>
+      <x:c r="H220"/>
+      <x:c r="I220"/>
+      <x:c r="J220"/>
+      <x:c r="K220" s="64"/>
+    </x:row>
+    <x:row r="221">
+      <x:c r="G221" s="57"/>
+      <x:c r="H221"/>
+      <x:c r="I221"/>
+      <x:c r="J221"/>
+      <x:c r="K221" s="64"/>
+    </x:row>
+    <x:row r="222">
+      <x:c r="G222" s="57"/>
+      <x:c r="H222"/>
+      <x:c r="I222"/>
+      <x:c r="J222"/>
+      <x:c r="K222" s="64"/>
+    </x:row>
+    <x:row r="223">
+      <x:c r="G223" s="57"/>
+      <x:c r="H223"/>
+      <x:c r="I223"/>
+      <x:c r="J223"/>
+      <x:c r="K223" s="64"/>
+    </x:row>
+    <x:row r="224">
+      <x:c r="G224" s="57"/>
+      <x:c r="H224"/>
+      <x:c r="I224"/>
+      <x:c r="J224"/>
+      <x:c r="K224" s="64"/>
+    </x:row>
+    <x:row r="225">
+      <x:c r="G225" s="57"/>
+      <x:c r="H225"/>
+      <x:c r="I225"/>
+      <x:c r="J225"/>
+      <x:c r="K225" s="64"/>
+    </x:row>
+    <x:row r="226">
+      <x:c r="G226" s="57"/>
+      <x:c r="H226"/>
+      <x:c r="I226"/>
+      <x:c r="J226"/>
+      <x:c r="K226" s="64"/>
+    </x:row>
+    <x:row r="227">
+      <x:c r="G227" s="57"/>
+      <x:c r="H227"/>
+      <x:c r="I227"/>
+      <x:c r="J227"/>
+      <x:c r="K227" s="64"/>
+    </x:row>
+    <x:row r="228">
+      <x:c r="G228" s="57"/>
+      <x:c r="H228"/>
+      <x:c r="I228"/>
+      <x:c r="J228"/>
+      <x:c r="K228" s="64"/>
+    </x:row>
+    <x:row r="229">
+      <x:c r="G229" s="57"/>
+      <x:c r="H229"/>
+      <x:c r="I229"/>
+      <x:c r="J229"/>
+      <x:c r="K229" s="64"/>
+    </x:row>
+    <x:row r="230">
+      <x:c r="G230" s="57"/>
+      <x:c r="H230"/>
+      <x:c r="I230"/>
+      <x:c r="J230"/>
+      <x:c r="K230" s="64"/>
+    </x:row>
+    <x:row r="231">
+      <x:c r="G231" s="57"/>
+      <x:c r="H231"/>
+      <x:c r="I231"/>
+      <x:c r="J231"/>
+      <x:c r="K231" s="64"/>
+    </x:row>
+    <x:row r="232">
+      <x:c r="G232" s="57"/>
+      <x:c r="H232"/>
+      <x:c r="I232"/>
+      <x:c r="J232"/>
+      <x:c r="K232" s="64"/>
+    </x:row>
+    <x:row r="233">
+      <x:c r="G233" s="57"/>
+      <x:c r="H233"/>
+      <x:c r="I233"/>
+      <x:c r="J233"/>
+      <x:c r="K233" s="64"/>
+    </x:row>
+    <x:row r="234">
+      <x:c r="G234" s="57"/>
+      <x:c r="H234"/>
+      <x:c r="I234"/>
+      <x:c r="J234"/>
+      <x:c r="K234" s="64"/>
+    </x:row>
+    <x:row r="235">
+      <x:c r="G235" s="57"/>
+      <x:c r="H235"/>
+      <x:c r="I235"/>
+      <x:c r="J235"/>
+      <x:c r="K235" s="64"/>
+    </x:row>
+    <x:row r="236">
+      <x:c r="G236" s="57"/>
+      <x:c r="H236"/>
+      <x:c r="I236"/>
+      <x:c r="J236"/>
+      <x:c r="K236" s="64"/>
+    </x:row>
+    <x:row r="237">
+      <x:c r="G237" s="57"/>
+      <x:c r="H237"/>
+      <x:c r="I237"/>
+      <x:c r="J237"/>
+      <x:c r="K237" s="64"/>
+    </x:row>
+    <x:row r="238">
+      <x:c r="G238" s="57"/>
+      <x:c r="H238"/>
+      <x:c r="I238"/>
+      <x:c r="J238"/>
+      <x:c r="K238" s="64"/>
+    </x:row>
+    <x:row r="239">
+      <x:c r="G239" s="57"/>
+      <x:c r="H239"/>
+      <x:c r="I239"/>
+      <x:c r="J239"/>
+      <x:c r="K239" s="64"/>
+    </x:row>
+    <x:row r="240">
+      <x:c r="G240" s="57"/>
+      <x:c r="H240"/>
+      <x:c r="I240"/>
+      <x:c r="J240"/>
+      <x:c r="K240" s="64"/>
+    </x:row>
+    <x:row r="241">
+      <x:c r="G241" s="57"/>
+      <x:c r="H241"/>
+      <x:c r="I241"/>
+      <x:c r="J241"/>
+      <x:c r="K241" s="64"/>
+    </x:row>
+    <x:row r="242">
+      <x:c r="G242" s="57"/>
+      <x:c r="H242"/>
+      <x:c r="I242"/>
+      <x:c r="J242"/>
+      <x:c r="K242" s="64"/>
+    </x:row>
+    <x:row r="243">
+      <x:c r="G243" s="57"/>
+      <x:c r="H243"/>
+      <x:c r="I243"/>
+      <x:c r="J243"/>
+      <x:c r="K243" s="64"/>
+    </x:row>
+    <x:row r="244">
+      <x:c r="G244" s="57"/>
+      <x:c r="H244"/>
+      <x:c r="I244"/>
+      <x:c r="J244"/>
+      <x:c r="K244" s="64"/>
+    </x:row>
+    <x:row r="245">
+      <x:c r="G245" s="57"/>
+      <x:c r="H245"/>
+      <x:c r="I245"/>
+      <x:c r="J245"/>
+      <x:c r="K245" s="64"/>
+    </x:row>
+    <x:row r="246">
+      <x:c r="G246" s="57"/>
+      <x:c r="H246"/>
+      <x:c r="I246"/>
+      <x:c r="J246"/>
+      <x:c r="K246" s="64"/>
+    </x:row>
+    <x:row r="247">
+      <x:c r="G247" s="57"/>
+      <x:c r="H247"/>
+      <x:c r="I247"/>
+      <x:c r="J247"/>
+      <x:c r="K247" s="64"/>
+    </x:row>
+    <x:row r="248">
+      <x:c r="G248" s="57"/>
+      <x:c r="H248"/>
+      <x:c r="I248"/>
+      <x:c r="J248"/>
+      <x:c r="K248" s="64"/>
+    </x:row>
+    <x:row r="249">
+      <x:c r="G249" s="57"/>
+      <x:c r="H249"/>
+      <x:c r="I249"/>
+      <x:c r="J249"/>
+      <x:c r="K249" s="64"/>
+    </x:row>
+    <x:row r="250">
+      <x:c r="G250" s="57"/>
+      <x:c r="H250"/>
+      <x:c r="I250"/>
+      <x:c r="J250"/>
+      <x:c r="K250" s="64"/>
+    </x:row>
+    <x:row r="251">
+      <x:c r="G251" s="57"/>
+      <x:c r="H251"/>
+      <x:c r="I251"/>
+      <x:c r="J251"/>
+      <x:c r="K251" s="64"/>
+    </x:row>
+    <x:row r="252">
+      <x:c r="G252" s="57"/>
+      <x:c r="H252"/>
+      <x:c r="I252"/>
+      <x:c r="J252"/>
+      <x:c r="K252" s="64"/>
+    </x:row>
+    <x:row r="253">
+      <x:c r="G253" s="57"/>
+      <x:c r="H253"/>
+      <x:c r="I253"/>
+      <x:c r="J253"/>
+      <x:c r="K253" s="64"/>
+    </x:row>
+    <x:row r="254">
+      <x:c r="G254" s="57"/>
+      <x:c r="H254"/>
+      <x:c r="I254"/>
+      <x:c r="J254"/>
+      <x:c r="K254" s="64"/>
+    </x:row>
+    <x:row r="255">
+      <x:c r="G255" s="57"/>
+      <x:c r="H255"/>
+      <x:c r="I255"/>
+      <x:c r="J255"/>
+      <x:c r="K255" s="64"/>
+    </x:row>
+    <x:row r="256">
+      <x:c r="G256" s="57"/>
+      <x:c r="H256"/>
+      <x:c r="I256"/>
+      <x:c r="J256"/>
+      <x:c r="K256" s="64"/>
+    </x:row>
+    <x:row r="257">
+      <x:c r="G257" s="57"/>
+      <x:c r="H257"/>
+      <x:c r="I257"/>
+      <x:c r="J257"/>
+      <x:c r="K257" s="64"/>
+    </x:row>
+    <x:row r="258">
+      <x:c r="G258" s="57"/>
+      <x:c r="H258"/>
+      <x:c r="I258"/>
+      <x:c r="J258"/>
+      <x:c r="K258" s="64"/>
+    </x:row>
+    <x:row r="259">
+      <x:c r="G259" s="57"/>
+      <x:c r="H259"/>
+      <x:c r="I259"/>
+      <x:c r="J259"/>
+      <x:c r="K259" s="64"/>
+    </x:row>
+    <x:row r="260">
+      <x:c r="G260" s="57"/>
+      <x:c r="H260"/>
+      <x:c r="I260"/>
+      <x:c r="J260"/>
+      <x:c r="K260" s="64"/>
+    </x:row>
+    <x:row r="261">
+      <x:c r="G261" s="57"/>
+      <x:c r="H261"/>
+      <x:c r="I261"/>
+      <x:c r="J261"/>
+      <x:c r="K261" s="64"/>
+    </x:row>
+    <x:row r="262">
+      <x:c r="G262" s="57"/>
+      <x:c r="H262"/>
+      <x:c r="I262"/>
+      <x:c r="J262"/>
+      <x:c r="K262" s="64"/>
+    </x:row>
+    <x:row r="263">
+      <x:c r="G263" s="57"/>
+      <x:c r="H263"/>
+      <x:c r="I263"/>
+      <x:c r="J263"/>
+      <x:c r="K263" s="64"/>
+    </x:row>
+    <x:row r="264">
+      <x:c r="G264" s="57"/>
+      <x:c r="H264"/>
+      <x:c r="I264"/>
+      <x:c r="J264"/>
+      <x:c r="K264" s="64"/>
+    </x:row>
+    <x:row r="265">
+      <x:c r="G265" s="57"/>
+      <x:c r="H265"/>
+      <x:c r="I265"/>
+      <x:c r="J265"/>
+      <x:c r="K265" s="64"/>
+    </x:row>
+    <x:row r="266">
+      <x:c r="G266" s="57"/>
+      <x:c r="H266"/>
+      <x:c r="I266"/>
+      <x:c r="J266"/>
+      <x:c r="K266" s="64"/>
+    </x:row>
+    <x:row r="267">
+      <x:c r="G267" s="57"/>
+      <x:c r="H267"/>
+      <x:c r="I267"/>
+      <x:c r="J267"/>
+      <x:c r="K267" s="64"/>
+    </x:row>
+    <x:row r="268">
+      <x:c r="G268" s="57"/>
+      <x:c r="H268"/>
+      <x:c r="I268"/>
+      <x:c r="J268"/>
+      <x:c r="K268" s="64"/>
+    </x:row>
+    <x:row r="269">
+      <x:c r="G269" s="57"/>
+      <x:c r="H269"/>
+      <x:c r="I269"/>
+      <x:c r="J269"/>
+      <x:c r="K269" s="64"/>
+    </x:row>
+    <x:row r="270">
+      <x:c r="G270" s="57"/>
+      <x:c r="H270"/>
+      <x:c r="I270"/>
+      <x:c r="J270"/>
+      <x:c r="K270" s="64"/>
+    </x:row>
+    <x:row r="271">
+      <x:c r="G271" s="57"/>
+      <x:c r="H271"/>
+      <x:c r="I271"/>
+      <x:c r="J271"/>
+      <x:c r="K271" s="64"/>
+    </x:row>
+    <x:row r="272">
+      <x:c r="G272" s="57"/>
+      <x:c r="H272"/>
+      <x:c r="I272"/>
+      <x:c r="J272"/>
+      <x:c r="K272" s="64"/>
+    </x:row>
+    <x:row r="273">
+      <x:c r="G273" s="57"/>
+      <x:c r="H273"/>
+      <x:c r="I273"/>
+      <x:c r="J273"/>
+      <x:c r="K273" s="64"/>
+    </x:row>
+    <x:row r="274">
+      <x:c r="G274" s="57"/>
+      <x:c r="H274"/>
+      <x:c r="I274"/>
+      <x:c r="J274"/>
+      <x:c r="K274" s="64"/>
+    </x:row>
+    <x:row r="275">
+      <x:c r="G275" s="57"/>
+      <x:c r="H275"/>
+      <x:c r="I275"/>
+      <x:c r="J275"/>
+      <x:c r="K275" s="64"/>
+    </x:row>
+    <x:row r="276">
+      <x:c r="G276" s="57"/>
+      <x:c r="H276"/>
+      <x:c r="I276"/>
+      <x:c r="J276"/>
+      <x:c r="K276" s="64"/>
+    </x:row>
+    <x:row r="277">
+      <x:c r="G277" s="57"/>
+      <x:c r="H277"/>
+      <x:c r="I277"/>
+      <x:c r="J277"/>
+      <x:c r="K277" s="64"/>
+    </x:row>
+    <x:row r="278">
+      <x:c r="G278" s="57"/>
+      <x:c r="H278"/>
+      <x:c r="I278"/>
+      <x:c r="J278"/>
+      <x:c r="K278" s="64"/>
+    </x:row>
+    <x:row r="279">
+      <x:c r="G279" s="57"/>
+      <x:c r="H279"/>
+      <x:c r="I279"/>
+      <x:c r="J279"/>
+      <x:c r="K279" s="64"/>
+    </x:row>
+    <x:row r="280">
+      <x:c r="G280" s="57"/>
+      <x:c r="H280"/>
+      <x:c r="I280"/>
+      <x:c r="J280"/>
+      <x:c r="K280" s="64"/>
+    </x:row>
+    <x:row r="281">
+      <x:c r="G281" s="57"/>
+      <x:c r="H281"/>
+      <x:c r="I281"/>
+      <x:c r="J281"/>
+      <x:c r="K281" s="64"/>
+    </x:row>
+    <x:row r="282">
+      <x:c r="G282" s="57"/>
+      <x:c r="H282"/>
+      <x:c r="I282"/>
+      <x:c r="J282"/>
+      <x:c r="K282" s="64"/>
+    </x:row>
+    <x:row r="283">
+      <x:c r="G283" s="57"/>
+      <x:c r="H283"/>
+      <x:c r="I283"/>
+      <x:c r="J283"/>
+      <x:c r="K283" s="64"/>
+    </x:row>
+    <x:row r="284">
+      <x:c r="G284" s="57"/>
+      <x:c r="H284"/>
+      <x:c r="I284"/>
+      <x:c r="J284"/>
+      <x:c r="K284" s="64"/>
+    </x:row>
+    <x:row r="285">
+      <x:c r="G285" s="57"/>
+      <x:c r="H285"/>
+      <x:c r="I285"/>
+      <x:c r="J285"/>
+      <x:c r="K285" s="64"/>
+    </x:row>
+    <x:row r="286">
+      <x:c r="G286" s="57"/>
+      <x:c r="H286"/>
+      <x:c r="I286"/>
+      <x:c r="J286"/>
+      <x:c r="K286" s="64"/>
+    </x:row>
+    <x:row r="287">
+      <x:c r="G287" s="57"/>
+      <x:c r="H287"/>
+      <x:c r="I287"/>
+      <x:c r="J287"/>
+      <x:c r="K287" s="64"/>
+    </x:row>
+    <x:row r="288">
+      <x:c r="G288" s="57"/>
+      <x:c r="H288"/>
+      <x:c r="I288"/>
+      <x:c r="J288"/>
+      <x:c r="K288" s="64"/>
+    </x:row>
+    <x:row r="289">
+      <x:c r="G289" s="57"/>
+      <x:c r="H289"/>
+      <x:c r="I289"/>
+      <x:c r="J289"/>
+      <x:c r="K289" s="64"/>
+    </x:row>
+    <x:row r="290">
+      <x:c r="G290" s="57"/>
+      <x:c r="H290"/>
+      <x:c r="I290"/>
+      <x:c r="J290"/>
+      <x:c r="K290" s="64"/>
+    </x:row>
+    <x:row r="291">
+      <x:c r="G291" s="57"/>
+      <x:c r="H291"/>
+      <x:c r="I291"/>
+      <x:c r="J291"/>
+      <x:c r="K291" s="64"/>
+    </x:row>
+    <x:row r="292">
+      <x:c r="G292" s="57"/>
+      <x:c r="H292"/>
+      <x:c r="I292"/>
+      <x:c r="J292"/>
+      <x:c r="K292" s="64"/>
+    </x:row>
+    <x:row r="293">
+      <x:c r="G293" s="57"/>
+      <x:c r="H293"/>
+      <x:c r="I293"/>
+      <x:c r="J293"/>
+      <x:c r="K293" s="64"/>
+    </x:row>
+    <x:row r="294">
+      <x:c r="G294" s="57"/>
+      <x:c r="H294"/>
+      <x:c r="I294"/>
+      <x:c r="J294"/>
+      <x:c r="K294" s="64"/>
+    </x:row>
+    <x:row r="295">
+      <x:c r="G295" s="57"/>
+      <x:c r="H295"/>
+      <x:c r="I295"/>
+      <x:c r="J295"/>
+      <x:c r="K295" s="64"/>
+    </x:row>
+    <x:row r="296">
+      <x:c r="G296" s="57"/>
+      <x:c r="H296"/>
+      <x:c r="I296"/>
+      <x:c r="J296"/>
+      <x:c r="K296" s="64"/>
+    </x:row>
+    <x:row r="297">
+      <x:c r="G297" s="57"/>
+      <x:c r="H297"/>
+      <x:c r="I297"/>
+      <x:c r="J297"/>
+      <x:c r="K297" s="64"/>
+    </x:row>
+    <x:row r="298">
+      <x:c r="G298" s="57"/>
+      <x:c r="H298"/>
+      <x:c r="I298"/>
+      <x:c r="J298"/>
+      <x:c r="K298" s="64"/>
+    </x:row>
+    <x:row r="299">
+      <x:c r="G299" s="57"/>
+      <x:c r="H299"/>
+      <x:c r="I299"/>
+      <x:c r="J299"/>
+      <x:c r="K299" s="64"/>
+    </x:row>
+    <x:row r="300">
+      <x:c r="G300" s="57"/>
+      <x:c r="H300"/>
+      <x:c r="I300"/>
+      <x:c r="J300"/>
+      <x:c r="K300" s="64"/>
+    </x:row>
+    <x:row r="301">
+      <x:c r="G301" s="57"/>
+      <x:c r="H301"/>
+      <x:c r="I301"/>
+      <x:c r="J301"/>
+      <x:c r="K301" s="64"/>
+    </x:row>
+    <x:row r="302">
+      <x:c r="G302" s="57"/>
+      <x:c r="H302"/>
+      <x:c r="I302"/>
+      <x:c r="J302"/>
+      <x:c r="K302" s="64"/>
+    </x:row>
+    <x:row r="303">
+      <x:c r="G303" s="57"/>
+      <x:c r="H303"/>
+      <x:c r="I303"/>
+      <x:c r="J303"/>
+      <x:c r="K303" s="64"/>
+    </x:row>
+    <x:row r="304">
+      <x:c r="G304" s="57"/>
+      <x:c r="H304"/>
+      <x:c r="I304"/>
+      <x:c r="J304"/>
+      <x:c r="K304" s="64"/>
+    </x:row>
+    <x:row r="305">
+      <x:c r="G305" s="57"/>
+      <x:c r="H305"/>
+      <x:c r="I305"/>
+      <x:c r="J305"/>
+      <x:c r="K305" s="64"/>
+    </x:row>
+    <x:row r="306">
+      <x:c r="G306" s="57"/>
+      <x:c r="H306"/>
+      <x:c r="I306"/>
+      <x:c r="J306"/>
+      <x:c r="K306" s="64"/>
+    </x:row>
+    <x:row r="307">
+      <x:c r="G307" s="57"/>
+      <x:c r="H307"/>
+      <x:c r="I307"/>
+      <x:c r="J307"/>
+      <x:c r="K307" s="64"/>
+    </x:row>
+    <x:row r="308">
+      <x:c r="G308" s="57"/>
+      <x:c r="H308"/>
+      <x:c r="I308"/>
+      <x:c r="J308"/>
+      <x:c r="K308" s="64"/>
+    </x:row>
+    <x:row r="309">
+      <x:c r="G309" s="57"/>
+      <x:c r="H309"/>
+      <x:c r="I309"/>
+      <x:c r="J309"/>
+      <x:c r="K309" s="64"/>
+    </x:row>
+    <x:row r="310">
+      <x:c r="G310" s="57"/>
+      <x:c r="H310"/>
+      <x:c r="I310"/>
+      <x:c r="J310"/>
+      <x:c r="K310" s="64"/>
+    </x:row>
+    <x:row r="311">
+      <x:c r="G311" s="57"/>
+      <x:c r="H311"/>
+      <x:c r="I311"/>
+      <x:c r="J311"/>
+      <x:c r="K311" s="64"/>
+    </x:row>
+    <x:row r="312">
+      <x:c r="G312" s="57"/>
+      <x:c r="H312"/>
+      <x:c r="I312"/>
+      <x:c r="J312"/>
+      <x:c r="K312" s="64"/>
+    </x:row>
+    <x:row r="313">
+      <x:c r="G313" s="57"/>
+      <x:c r="H313"/>
+      <x:c r="I313"/>
+      <x:c r="J313"/>
+      <x:c r="K313" s="64"/>
+    </x:row>
+    <x:row r="314">
+      <x:c r="G314" s="57"/>
+      <x:c r="H314"/>
+      <x:c r="I314"/>
+      <x:c r="J314"/>
+      <x:c r="K314" s="64"/>
+    </x:row>
+    <x:row r="315">
+      <x:c r="G315" s="57"/>
+      <x:c r="H315"/>
+      <x:c r="I315"/>
+      <x:c r="J315"/>
+      <x:c r="K315" s="64"/>
+    </x:row>
+    <x:row r="316">
+      <x:c r="G316" s="57"/>
+      <x:c r="H316"/>
+      <x:c r="I316"/>
+      <x:c r="J316"/>
+      <x:c r="K316" s="64"/>
+    </x:row>
+    <x:row r="317">
+      <x:c r="G317" s="57"/>
+      <x:c r="H317"/>
+      <x:c r="I317"/>
+      <x:c r="J317"/>
+      <x:c r="K317" s="64"/>
+    </x:row>
+    <x:row r="318">
+      <x:c r="G318" s="57"/>
+      <x:c r="H318"/>
+      <x:c r="I318"/>
+      <x:c r="J318"/>
+      <x:c r="K318" s="64"/>
+    </x:row>
+    <x:row r="319">
+      <x:c r="G319" s="57"/>
+      <x:c r="H319"/>
+      <x:c r="I319"/>
+      <x:c r="J319"/>
+      <x:c r="K319" s="64"/>
+    </x:row>
+    <x:row r="320">
+      <x:c r="G320" s="57"/>
+      <x:c r="H320"/>
+      <x:c r="I320"/>
+      <x:c r="J320"/>
+      <x:c r="K320" s="64"/>
+    </x:row>
+    <x:row r="321">
+      <x:c r="G321" s="57"/>
+      <x:c r="H321"/>
+      <x:c r="I321"/>
+      <x:c r="J321"/>
+      <x:c r="K321" s="64"/>
+    </x:row>
+    <x:row r="322">
+      <x:c r="G322" s="57"/>
+      <x:c r="H322"/>
+      <x:c r="I322"/>
+      <x:c r="J322"/>
+      <x:c r="K322" s="64"/>
+    </x:row>
+    <x:row r="323">
+      <x:c r="G323" s="57"/>
+      <x:c r="H323"/>
+      <x:c r="I323"/>
+      <x:c r="J323"/>
+      <x:c r="K323" s="64"/>
+    </x:row>
+    <x:row r="324">
+      <x:c r="G324" s="57"/>
+      <x:c r="H324"/>
+      <x:c r="I324"/>
+      <x:c r="J324"/>
+      <x:c r="K324" s="64"/>
+    </x:row>
+    <x:row r="325">
+      <x:c r="G325" s="57"/>
+      <x:c r="H325"/>
+      <x:c r="I325"/>
+      <x:c r="J325"/>
+      <x:c r="K325" s="64"/>
+    </x:row>
+    <x:row r="326">
+      <x:c r="G326" s="57"/>
+      <x:c r="H326"/>
+      <x:c r="I326"/>
+      <x:c r="J326"/>
+      <x:c r="K326" s="64"/>
+    </x:row>
+    <x:row r="327">
+      <x:c r="G327" s="57"/>
+      <x:c r="H327"/>
+      <x:c r="I327"/>
+      <x:c r="J327"/>
+      <x:c r="K327" s="64"/>
+    </x:row>
+    <x:row r="328">
+      <x:c r="G328" s="57"/>
+      <x:c r="H328"/>
+      <x:c r="I328"/>
+      <x:c r="J328"/>
+      <x:c r="K328" s="64"/>
+    </x:row>
+    <x:row r="329">
+      <x:c r="G329" s="57"/>
+      <x:c r="H329"/>
+      <x:c r="I329"/>
+      <x:c r="J329"/>
+      <x:c r="K329" s="64"/>
+    </x:row>
+    <x:row r="330">
+      <x:c r="G330" s="57"/>
+      <x:c r="H330"/>
+      <x:c r="I330"/>
+      <x:c r="J330"/>
+      <x:c r="K330" s="64"/>
+    </x:row>
+    <x:row r="331">
+      <x:c r="G331" s="57"/>
+      <x:c r="H331"/>
+      <x:c r="I331"/>
+      <x:c r="J331"/>
+      <x:c r="K331" s="64"/>
+    </x:row>
+    <x:row r="332">
+      <x:c r="G332" s="57"/>
+      <x:c r="H332"/>
+      <x:c r="I332"/>
+      <x:c r="J332"/>
+      <x:c r="K332" s="64"/>
+    </x:row>
+    <x:row r="333">
+      <x:c r="G333" s="57"/>
+      <x:c r="H333"/>
+      <x:c r="I333"/>
+      <x:c r="J333"/>
+      <x:c r="K333" s="64"/>
+    </x:row>
+    <x:row r="334">
+      <x:c r="G334" s="57"/>
+      <x:c r="H334"/>
+      <x:c r="I334"/>
+      <x:c r="J334"/>
+      <x:c r="K334" s="64"/>
+    </x:row>
+    <x:row r="335">
+      <x:c r="G335" s="57"/>
+      <x:c r="H335"/>
+      <x:c r="I335"/>
+      <x:c r="J335"/>
+      <x:c r="K335" s="64"/>
+    </x:row>
+    <x:row r="336">
+      <x:c r="G336" s="57"/>
+      <x:c r="H336"/>
+      <x:c r="I336"/>
+      <x:c r="J336"/>
+      <x:c r="K336" s="64"/>
+    </x:row>
+    <x:row r="337">
+      <x:c r="G337" s="57"/>
+      <x:c r="H337"/>
+      <x:c r="I337"/>
+      <x:c r="J337"/>
+      <x:c r="K337" s="64"/>
+    </x:row>
+    <x:row r="338">
+      <x:c r="G338" s="57"/>
+      <x:c r="H338"/>
+      <x:c r="I338"/>
+      <x:c r="J338"/>
+      <x:c r="K338" s="64"/>
+    </x:row>
+    <x:row r="339">
+      <x:c r="G339" s="57"/>
+      <x:c r="H339"/>
+      <x:c r="I339"/>
+      <x:c r="J339"/>
+      <x:c r="K339" s="64"/>
+    </x:row>
+    <x:row r="340">
+      <x:c r="G340" s="57"/>
+      <x:c r="H340"/>
+      <x:c r="I340"/>
+      <x:c r="J340"/>
+      <x:c r="K340" s="64"/>
+    </x:row>
+    <x:row r="341">
+      <x:c r="G341" s="57"/>
+      <x:c r="H341"/>
+      <x:c r="I341"/>
+      <x:c r="J341"/>
+      <x:c r="K341" s="64"/>
+    </x:row>
+    <x:row r="342">
+      <x:c r="G342" s="57"/>
+      <x:c r="H342"/>
+      <x:c r="I342"/>
+      <x:c r="J342"/>
+      <x:c r="K342" s="64"/>
+    </x:row>
+    <x:row r="343">
+      <x:c r="G343" s="57"/>
+      <x:c r="H343"/>
+      <x:c r="I343"/>
+      <x:c r="J343"/>
+      <x:c r="K343" s="64"/>
+    </x:row>
+    <x:row r="344">
+      <x:c r="G344" s="57"/>
+      <x:c r="H344"/>
+      <x:c r="I344"/>
+      <x:c r="J344"/>
+      <x:c r="K344" s="64"/>
+    </x:row>
+    <x:row r="345">
+      <x:c r="G345" s="57"/>
+      <x:c r="H345"/>
+      <x:c r="I345"/>
+      <x:c r="J345"/>
+      <x:c r="K345" s="64"/>
+    </x:row>
+    <x:row r="346">
+      <x:c r="G346" s="57"/>
+      <x:c r="H346"/>
+      <x:c r="I346"/>
+      <x:c r="J346"/>
+      <x:c r="K346" s="64"/>
+    </x:row>
+    <x:row r="347">
+      <x:c r="G347" s="57"/>
+      <x:c r="H347"/>
+      <x:c r="I347"/>
+      <x:c r="J347"/>
+      <x:c r="K347" s="64"/>
+    </x:row>
+    <x:row r="348">
+      <x:c r="G348" s="57"/>
+      <x:c r="H348"/>
+      <x:c r="I348"/>
+      <x:c r="J348"/>
+      <x:c r="K348" s="64"/>
+    </x:row>
+    <x:row r="349">
+      <x:c r="G349" s="57"/>
+      <x:c r="H349"/>
+      <x:c r="I349"/>
+      <x:c r="J349"/>
+      <x:c r="K349" s="64"/>
+    </x:row>
+    <x:row r="350">
+      <x:c r="G350" s="57"/>
+      <x:c r="H350"/>
+      <x:c r="I350"/>
+      <x:c r="J350"/>
+      <x:c r="K350" s="64"/>
+    </x:row>
+    <x:row r="351">
+      <x:c r="G351" s="57"/>
+      <x:c r="H351"/>
+      <x:c r="I351"/>
+      <x:c r="J351"/>
+      <x:c r="K351" s="64"/>
+    </x:row>
+    <x:row r="352">
+      <x:c r="G352" s="57"/>
+      <x:c r="H352"/>
+      <x:c r="I352"/>
+      <x:c r="J352"/>
+      <x:c r="K352" s="64"/>
+    </x:row>
+    <x:row r="353">
+      <x:c r="G353" s="57"/>
+      <x:c r="H353"/>
+      <x:c r="I353"/>
+      <x:c r="J353"/>
+      <x:c r="K353" s="64"/>
+    </x:row>
+    <x:row r="354">
+      <x:c r="G354" s="57"/>
+      <x:c r="H354"/>
+      <x:c r="I354"/>
+      <x:c r="J354"/>
+      <x:c r="K354" s="64"/>
+    </x:row>
+    <x:row r="355">
+      <x:c r="G355" s="57"/>
+      <x:c r="H355"/>
+      <x:c r="I355"/>
+      <x:c r="J355"/>
+      <x:c r="K355" s="64"/>
+    </x:row>
+    <x:row r="356">
+      <x:c r="G356" s="57"/>
+      <x:c r="H356"/>
+      <x:c r="I356"/>
+      <x:c r="J356"/>
+      <x:c r="K356" s="64"/>
+    </x:row>
+    <x:row r="357">
+      <x:c r="G357" s="57"/>
+      <x:c r="H357"/>
+      <x:c r="I357"/>
+      <x:c r="J357"/>
+      <x:c r="K357" s="64"/>
+    </x:row>
+    <x:row r="358">
+      <x:c r="G358" s="57"/>
+      <x:c r="H358"/>
+      <x:c r="I358"/>
+      <x:c r="J358"/>
+      <x:c r="K358" s="64"/>
+    </x:row>
+    <x:row r="359">
+      <x:c r="G359" s="57"/>
+      <x:c r="H359"/>
+      <x:c r="I359"/>
+      <x:c r="J359"/>
+      <x:c r="K359" s="64"/>
+    </x:row>
+    <x:row r="360">
+      <x:c r="G360" s="57"/>
+      <x:c r="H360"/>
+      <x:c r="I360"/>
+      <x:c r="J360"/>
+      <x:c r="K360" s="64"/>
+    </x:row>
+    <x:row r="361">
+      <x:c r="G361" s="57"/>
+      <x:c r="H361"/>
+      <x:c r="I361"/>
+      <x:c r="J361"/>
+      <x:c r="K361" s="64"/>
+    </x:row>
+    <x:row r="362">
+      <x:c r="G362" s="57"/>
+      <x:c r="H362"/>
+      <x:c r="I362"/>
+      <x:c r="J362"/>
+      <x:c r="K362" s="64"/>
+    </x:row>
+    <x:row r="363">
+      <x:c r="G363" s="57"/>
+      <x:c r="H363"/>
+      <x:c r="I363"/>
+      <x:c r="J363"/>
+      <x:c r="K363" s="64"/>
+    </x:row>
+    <x:row r="364">
+      <x:c r="G364" s="57"/>
+      <x:c r="H364"/>
+      <x:c r="I364"/>
+      <x:c r="J364"/>
+      <x:c r="K364" s="64"/>
+    </x:row>
+    <x:row r="365">
+      <x:c r="G365" s="57"/>
+      <x:c r="H365"/>
+      <x:c r="I365"/>
+      <x:c r="J365"/>
+      <x:c r="K365" s="64"/>
+    </x:row>
+    <x:row r="366">
+      <x:c r="G366" s="57"/>
+      <x:c r="H366"/>
+      <x:c r="I366"/>
+      <x:c r="J366"/>
+      <x:c r="K366" s="64"/>
+    </x:row>
+    <x:row r="367">
+      <x:c r="G367" s="57"/>
+      <x:c r="H367"/>
+      <x:c r="I367"/>
+      <x:c r="J367"/>
+      <x:c r="K367" s="64"/>
+    </x:row>
+    <x:row r="368">
+      <x:c r="G368" s="57"/>
+      <x:c r="H368"/>
+      <x:c r="I368"/>
+      <x:c r="J368"/>
+      <x:c r="K368" s="64"/>
+    </x:row>
+    <x:row r="369">
+      <x:c r="G369" s="57"/>
+      <x:c r="H369"/>
+      <x:c r="I369"/>
+      <x:c r="J369"/>
+      <x:c r="K369" s="64"/>
+    </x:row>
+    <x:row r="370">
+      <x:c r="G370" s="57"/>
+      <x:c r="H370"/>
+      <x:c r="I370"/>
+      <x:c r="J370"/>
+      <x:c r="K370" s="64"/>
+    </x:row>
+    <x:row r="371">
+      <x:c r="G371" s="57"/>
+      <x:c r="H371"/>
+      <x:c r="I371"/>
+      <x:c r="J371"/>
+      <x:c r="K371" s="64"/>
+    </x:row>
+    <x:row r="372">
+      <x:c r="G372" s="57"/>
+      <x:c r="H372"/>
+      <x:c r="I372"/>
+      <x:c r="J372"/>
+      <x:c r="K372" s="64"/>
+    </x:row>
+    <x:row r="373">
+      <x:c r="G373" s="57"/>
+      <x:c r="H373"/>
+      <x:c r="I373"/>
+      <x:c r="J373"/>
+      <x:c r="K373" s="64"/>
+    </x:row>
+    <x:row r="374">
+      <x:c r="G374" s="57"/>
+      <x:c r="H374"/>
+      <x:c r="I374"/>
+      <x:c r="J374"/>
+      <x:c r="K374" s="64"/>
+    </x:row>
+    <x:row r="375">
+      <x:c r="G375" s="57"/>
+      <x:c r="H375"/>
+      <x:c r="I375"/>
+      <x:c r="J375"/>
+      <x:c r="K375" s="64"/>
+    </x:row>
+    <x:row r="376">
+      <x:c r="G376" s="57"/>
+      <x:c r="H376"/>
+      <x:c r="I376"/>
+      <x:c r="J376"/>
+      <x:c r="K376" s="64"/>
+    </x:row>
+    <x:row r="377">
+      <x:c r="G377" s="57"/>
+      <x:c r="H377"/>
+      <x:c r="I377"/>
+      <x:c r="J377"/>
+      <x:c r="K377" s="64"/>
+    </x:row>
+    <x:row r="378">
+      <x:c r="G378" s="57"/>
+      <x:c r="H378"/>
+      <x:c r="I378"/>
+      <x:c r="J378"/>
+      <x:c r="K378" s="64"/>
+    </x:row>
+    <x:row r="379">
+      <x:c r="G379" s="57"/>
+      <x:c r="H379"/>
+      <x:c r="I379"/>
+      <x:c r="J379"/>
+      <x:c r="K379" s="64"/>
+    </x:row>
+    <x:row r="380">
+      <x:c r="G380" s="57"/>
+      <x:c r="H380"/>
+      <x:c r="I380"/>
+      <x:c r="J380"/>
+      <x:c r="K380" s="64"/>
+    </x:row>
+    <x:row r="381">
+      <x:c r="G381" s="57"/>
+      <x:c r="H381"/>
+      <x:c r="I381"/>
+      <x:c r="J381"/>
+      <x:c r="K381" s="64"/>
+    </x:row>
+    <x:row r="382">
+      <x:c r="G382" s="57"/>
+      <x:c r="H382"/>
+      <x:c r="I382"/>
+      <x:c r="J382"/>
+      <x:c r="K382" s="64"/>
+    </x:row>
+    <x:row r="383">
+      <x:c r="G383" s="57"/>
+      <x:c r="H383"/>
+      <x:c r="I383"/>
+      <x:c r="J383"/>
+      <x:c r="K383" s="64"/>
+    </x:row>
+    <x:row r="384">
+      <x:c r="G384" s="57"/>
+      <x:c r="H384"/>
+      <x:c r="I384"/>
+      <x:c r="J384"/>
+      <x:c r="K384" s="64"/>
+    </x:row>
+    <x:row r="385">
+      <x:c r="G385" s="57"/>
+      <x:c r="H385"/>
+      <x:c r="I385"/>
+      <x:c r="J385"/>
+      <x:c r="K385" s="64"/>
+    </x:row>
+    <x:row r="386">
+      <x:c r="G386" s="57"/>
+      <x:c r="H386"/>
+      <x:c r="I386"/>
+      <x:c r="J386"/>
+      <x:c r="K386" s="64"/>
+    </x:row>
+    <x:row r="387">
+      <x:c r="G387" s="57"/>
+      <x:c r="H387"/>
+      <x:c r="I387"/>
+      <x:c r="J387"/>
+      <x:c r="K387" s="64"/>
+    </x:row>
+    <x:row r="388">
+      <x:c r="G388" s="57"/>
+      <x:c r="H388"/>
+      <x:c r="I388"/>
+      <x:c r="J388"/>
+      <x:c r="K388" s="64"/>
+    </x:row>
+    <x:row r="389">
+      <x:c r="G389" s="57"/>
+      <x:c r="H389"/>
+      <x:c r="I389"/>
+      <x:c r="J389"/>
+      <x:c r="K389" s="64"/>
+    </x:row>
+    <x:row r="390">
+      <x:c r="G390" s="57"/>
+      <x:c r="H390"/>
+      <x:c r="I390"/>
+      <x:c r="J390"/>
+      <x:c r="K390" s="64"/>
+    </x:row>
+    <x:row r="391">
+      <x:c r="G391" s="57"/>
+      <x:c r="H391"/>
+      <x:c r="I391"/>
+      <x:c r="J391"/>
+      <x:c r="K391" s="64"/>
+    </x:row>
+    <x:row r="392">
+      <x:c r="G392" s="57"/>
+      <x:c r="H392"/>
+      <x:c r="I392"/>
+      <x:c r="J392"/>
+      <x:c r="K392" s="64"/>
+    </x:row>
+    <x:row r="393">
+      <x:c r="G393" s="57"/>
+      <x:c r="H393"/>
+      <x:c r="I393"/>
+      <x:c r="J393"/>
+      <x:c r="K393" s="64"/>
+    </x:row>
+    <x:row r="394">
+      <x:c r="G394" s="57"/>
+      <x:c r="H394"/>
+      <x:c r="I394"/>
+      <x:c r="J394"/>
+      <x:c r="K394" s="64"/>
+    </x:row>
+    <x:row r="395">
+      <x:c r="G395" s="57"/>
+      <x:c r="H395"/>
+      <x:c r="I395"/>
+      <x:c r="J395"/>
+      <x:c r="K395" s="64"/>
+    </x:row>
+    <x:row r="396">
+      <x:c r="G396" s="57"/>
+      <x:c r="H396"/>
+      <x:c r="I396"/>
+      <x:c r="J396"/>
+      <x:c r="K396" s="64"/>
+    </x:row>
+    <x:row r="397">
+      <x:c r="G397" s="57"/>
+      <x:c r="H397"/>
+      <x:c r="I397"/>
+      <x:c r="J397"/>
+      <x:c r="K397" s="64"/>
+    </x:row>
+    <x:row r="398">
+      <x:c r="G398" s="57"/>
+      <x:c r="H398"/>
+      <x:c r="I398"/>
+      <x:c r="J398"/>
+      <x:c r="K398" s="64"/>
+    </x:row>
+    <x:row r="399">
+      <x:c r="G399" s="57"/>
+      <x:c r="H399"/>
+      <x:c r="I399"/>
+      <x:c r="J399"/>
+      <x:c r="K399" s="64"/>
+    </x:row>
+    <x:row r="400">
+      <x:c r="G400" s="57"/>
+      <x:c r="H400"/>
+      <x:c r="I400"/>
+      <x:c r="J400"/>
+      <x:c r="K400" s="64"/>
+    </x:row>
+    <x:row r="401">
+      <x:c r="G401" s="57"/>
+      <x:c r="H401"/>
+      <x:c r="I401"/>
+      <x:c r="J401"/>
+      <x:c r="K401" s="64"/>
+    </x:row>
+    <x:row r="402">
+      <x:c r="G402" s="57"/>
+      <x:c r="H402"/>
+      <x:c r="I402"/>
+      <x:c r="J402"/>
+      <x:c r="K402" s="64"/>
+    </x:row>
+    <x:row r="403">
+      <x:c r="G403" s="57"/>
+      <x:c r="H403"/>
+      <x:c r="I403"/>
+      <x:c r="J403"/>
+      <x:c r="K403" s="64"/>
+    </x:row>
+    <x:row r="404">
+      <x:c r="G404" s="57"/>
+      <x:c r="H404"/>
+      <x:c r="I404"/>
+      <x:c r="J404"/>
+      <x:c r="K404" s="64"/>
+    </x:row>
+    <x:row r="405">
+      <x:c r="G405" s="57"/>
+      <x:c r="H405"/>
+      <x:c r="I405"/>
+      <x:c r="J405"/>
+      <x:c r="K405" s="64"/>
+    </x:row>
+    <x:row r="406">
+      <x:c r="G406" s="57"/>
+      <x:c r="H406"/>
+      <x:c r="I406"/>
+      <x:c r="J406"/>
+      <x:c r="K406" s="64"/>
+    </x:row>
+    <x:row r="407">
+      <x:c r="G407" s="57"/>
+      <x:c r="H407"/>
+      <x:c r="I407"/>
+      <x:c r="J407"/>
+      <x:c r="K407" s="64"/>
+    </x:row>
+    <x:row r="408">
+      <x:c r="G408" s="57"/>
+      <x:c r="H408"/>
+      <x:c r="I408"/>
+      <x:c r="J408"/>
+      <x:c r="K408" s="64"/>
+    </x:row>
+    <x:row r="409">
+      <x:c r="G409" s="57"/>
+      <x:c r="H409"/>
+      <x:c r="I409"/>
+      <x:c r="J409"/>
+      <x:c r="K409" s="64"/>
+    </x:row>
+    <x:row r="410">
+      <x:c r="G410" s="57"/>
+      <x:c r="H410"/>
+      <x:c r="I410"/>
+      <x:c r="J410"/>
+      <x:c r="K410" s="64"/>
+    </x:row>
+    <x:row r="411">
+      <x:c r="G411" s="57"/>
+      <x:c r="H411"/>
+      <x:c r="I411"/>
+      <x:c r="J411"/>
+      <x:c r="K411" s="64"/>
+    </x:row>
+    <x:row r="412">
+      <x:c r="G412" s="57"/>
+      <x:c r="H412"/>
+      <x:c r="I412"/>
+      <x:c r="J412"/>
+      <x:c r="K412" s="64"/>
+    </x:row>
+    <x:row r="413">
+      <x:c r="G413" s="57"/>
+      <x:c r="H413"/>
+      <x:c r="I413"/>
+      <x:c r="J413"/>
+      <x:c r="K413" s="64"/>
+    </x:row>
+    <x:row r="414">
+      <x:c r="G414" s="57"/>
+      <x:c r="H414"/>
+      <x:c r="I414"/>
+      <x:c r="J414"/>
+      <x:c r="K414" s="64"/>
+    </x:row>
+    <x:row r="415">
+      <x:c r="G415" s="57"/>
+      <x:c r="H415"/>
+      <x:c r="I415"/>
+      <x:c r="J415"/>
+      <x:c r="K415" s="64"/>
+    </x:row>
+    <x:row r="416">
+      <x:c r="G416" s="57"/>
+      <x:c r="H416"/>
+      <x:c r="I416"/>
+      <x:c r="J416"/>
+      <x:c r="K416" s="64"/>
+    </x:row>
+    <x:row r="417">
+      <x:c r="G417" s="57"/>
+      <x:c r="H417"/>
+      <x:c r="I417"/>
+      <x:c r="J417"/>
+      <x:c r="K417" s="64"/>
+    </x:row>
+    <x:row r="418">
+      <x:c r="G418" s="57"/>
+      <x:c r="H418"/>
+      <x:c r="I418"/>
+      <x:c r="J418"/>
+      <x:c r="K418" s="64"/>
+    </x:row>
+    <x:row r="419">
+      <x:c r="G419" s="57"/>
+      <x:c r="H419"/>
+      <x:c r="I419"/>
+      <x:c r="J419"/>
+      <x:c r="K419" s="64"/>
+    </x:row>
+    <x:row r="420">
+      <x:c r="G420" s="57"/>
+      <x:c r="H420"/>
+      <x:c r="I420"/>
+      <x:c r="J420"/>
+      <x:c r="K420" s="64"/>
+    </x:row>
+    <x:row r="421">
+      <x:c r="G421" s="57"/>
+      <x:c r="H421"/>
+      <x:c r="I421"/>
+      <x:c r="J421"/>
+      <x:c r="K421" s="64"/>
+    </x:row>
+    <x:row r="422">
+      <x:c r="G422" s="57"/>
+      <x:c r="H422"/>
+      <x:c r="I422"/>
+      <x:c r="J422"/>
+      <x:c r="K422" s="64"/>
+    </x:row>
+    <x:row r="423">
+      <x:c r="G423" s="57"/>
+      <x:c r="H423"/>
+      <x:c r="I423"/>
+      <x:c r="J423"/>
+      <x:c r="K423" s="64"/>
+    </x:row>
+    <x:row r="424">
+      <x:c r="G424" s="57"/>
+      <x:c r="H424"/>
+      <x:c r="I424"/>
+      <x:c r="J424"/>
+      <x:c r="K424" s="64"/>
+    </x:row>
+    <x:row r="425">
+      <x:c r="G425" s="57"/>
+      <x:c r="H425"/>
+      <x:c r="I425"/>
+      <x:c r="J425"/>
+      <x:c r="K425" s="64"/>
+    </x:row>
+    <x:row r="426">
+      <x:c r="G426" s="57"/>
+      <x:c r="H426"/>
+      <x:c r="I426"/>
+      <x:c r="J426"/>
+      <x:c r="K426" s="64"/>
+    </x:row>
+    <x:row r="427">
+      <x:c r="G427" s="57"/>
+      <x:c r="H427"/>
+      <x:c r="I427"/>
+      <x:c r="J427"/>
+      <x:c r="K427" s="64"/>
+    </x:row>
+    <x:row r="428">
+      <x:c r="G428" s="57"/>
+      <x:c r="H428"/>
+      <x:c r="I428"/>
+      <x:c r="J428"/>
+      <x:c r="K428" s="64"/>
+    </x:row>
+    <x:row r="429">
+      <x:c r="G429" s="57"/>
+      <x:c r="H429"/>
+      <x:c r="I429"/>
+      <x:c r="J429"/>
+      <x:c r="K429" s="64"/>
+    </x:row>
+    <x:row r="430">
+      <x:c r="G430" s="57"/>
+      <x:c r="H430"/>
+      <x:c r="I430"/>
+      <x:c r="J430"/>
+      <x:c r="K430" s="64"/>
+    </x:row>
+    <x:row r="431">
+      <x:c r="G431" s="57"/>
+      <x:c r="H431"/>
+      <x:c r="I431"/>
+      <x:c r="J431"/>
+      <x:c r="K431" s="64"/>
+    </x:row>
+    <x:row r="432">
+      <x:c r="G432" s="57"/>
+      <x:c r="H432"/>
+      <x:c r="I432"/>
+      <x:c r="J432"/>
+      <x:c r="K432" s="64"/>
+    </x:row>
+    <x:row r="433">
+      <x:c r="G433" s="57"/>
+      <x:c r="H433"/>
+      <x:c r="I433"/>
+      <x:c r="J433"/>
+      <x:c r="K433" s="64"/>
+    </x:row>
+    <x:row r="434">
+      <x:c r="G434" s="57"/>
+      <x:c r="H434"/>
+      <x:c r="I434"/>
+      <x:c r="J434"/>
+      <x:c r="K434" s="64"/>
+    </x:row>
+    <x:row r="435">
+      <x:c r="G435" s="57"/>
+      <x:c r="H435"/>
+      <x:c r="I435"/>
+      <x:c r="J435"/>
+      <x:c r="K435" s="64"/>
+    </x:row>
+    <x:row r="436">
+      <x:c r="G436" s="57"/>
+      <x:c r="H436"/>
+      <x:c r="I436"/>
+      <x:c r="J436"/>
+      <x:c r="K436" s="64"/>
+    </x:row>
+    <x:row r="437">
+      <x:c r="G437" s="57"/>
+      <x:c r="H437"/>
+      <x:c r="I437"/>
+      <x:c r="J437"/>
+      <x:c r="K437" s="64"/>
+    </x:row>
+    <x:row r="438">
+      <x:c r="G438" s="57"/>
+      <x:c r="H438"/>
+      <x:c r="I438"/>
+      <x:c r="J438"/>
+      <x:c r="K438" s="64"/>
+    </x:row>
+    <x:row r="439">
+      <x:c r="G439" s="57"/>
+      <x:c r="H439"/>
+      <x:c r="I439"/>
+      <x:c r="J439"/>
+      <x:c r="K439" s="64"/>
+    </x:row>
+    <x:row r="440">
+      <x:c r="G440" s="57"/>
+      <x:c r="H440"/>
+      <x:c r="I440"/>
+      <x:c r="J440"/>
+      <x:c r="K440" s="64"/>
+    </x:row>
+    <x:row r="441">
+      <x:c r="G441" s="57"/>
+      <x:c r="H441"/>
+      <x:c r="I441"/>
+      <x:c r="J441"/>
+      <x:c r="K441" s="64"/>
+    </x:row>
+    <x:row r="442">
+      <x:c r="G442" s="57"/>
+      <x:c r="H442"/>
+      <x:c r="I442"/>
+      <x:c r="J442"/>
+      <x:c r="K442" s="64"/>
+    </x:row>
+    <x:row r="443">
+      <x:c r="G443" s="57"/>
+      <x:c r="H443"/>
+      <x:c r="I443"/>
+      <x:c r="J443"/>
+      <x:c r="K443" s="64"/>
+    </x:row>
+    <x:row r="444">
+      <x:c r="G444" s="57"/>
+      <x:c r="H444"/>
+      <x:c r="I444"/>
+      <x:c r="J444"/>
+      <x:c r="K444" s="64"/>
+    </x:row>
+    <x:row r="445">
+      <x:c r="G445" s="57"/>
+      <x:c r="H445"/>
+      <x:c r="I445"/>
+      <x:c r="J445"/>
+      <x:c r="K445" s="64"/>
+    </x:row>
+    <x:row r="446">
+      <x:c r="G446" s="57"/>
+      <x:c r="H446"/>
+      <x:c r="I446"/>
+      <x:c r="J446"/>
+      <x:c r="K446" s="64"/>
+    </x:row>
+    <x:row r="447">
+      <x:c r="G447" s="57"/>
+      <x:c r="H447"/>
+      <x:c r="I447"/>
+      <x:c r="J447"/>
+      <x:c r="K447" s="64"/>
+    </x:row>
+    <x:row r="448">
+      <x:c r="G448" s="57"/>
+      <x:c r="H448"/>
+      <x:c r="I448"/>
+      <x:c r="J448"/>
+      <x:c r="K448" s="64"/>
+    </x:row>
+    <x:row r="449">
+      <x:c r="G449" s="57"/>
+      <x:c r="H449"/>
+      <x:c r="I449"/>
+      <x:c r="J449"/>
+      <x:c r="K449" s="64"/>
+    </x:row>
+    <x:row r="450">
+      <x:c r="G450" s="57"/>
+      <x:c r="H450"/>
+      <x:c r="I450"/>
+      <x:c r="J450"/>
+      <x:c r="K450" s="64"/>
+    </x:row>
+    <x:row r="451">
+      <x:c r="G451" s="57"/>
+      <x:c r="H451"/>
+      <x:c r="I451"/>
+      <x:c r="J451"/>
+      <x:c r="K451" s="64"/>
+    </x:row>
+    <x:row r="452">
+      <x:c r="G452" s="57"/>
+      <x:c r="H452"/>
+      <x:c r="I452"/>
+      <x:c r="J452"/>
+      <x:c r="K452" s="64"/>
+    </x:row>
+    <x:row r="453">
+      <x:c r="G453" s="57"/>
+      <x:c r="H453"/>
+      <x:c r="I453"/>
+      <x:c r="J453"/>
+      <x:c r="K453" s="64"/>
+    </x:row>
+    <x:row r="454">
+      <x:c r="G454" s="57"/>
+      <x:c r="H454"/>
+      <x:c r="I454"/>
+      <x:c r="J454"/>
+      <x:c r="K454" s="64"/>
+    </x:row>
+    <x:row r="455">
+      <x:c r="G455" s="57"/>
+      <x:c r="H455"/>
+      <x:c r="I455"/>
+      <x:c r="J455"/>
+      <x:c r="K455" s="64"/>
+    </x:row>
+    <x:row r="456">
+      <x:c r="G456" s="57"/>
+      <x:c r="H456"/>
+      <x:c r="I456"/>
+      <x:c r="J456"/>
+      <x:c r="K456" s="64"/>
+    </x:row>
+    <x:row r="457">
+      <x:c r="G457" s="57"/>
+      <x:c r="H457"/>
+      <x:c r="I457"/>
+      <x:c r="J457"/>
+      <x:c r="K457" s="64"/>
+    </x:row>
+    <x:row r="458">
+      <x:c r="G458" s="57"/>
+      <x:c r="H458"/>
+      <x:c r="I458"/>
+      <x:c r="J458"/>
+      <x:c r="K458" s="64"/>
+    </x:row>
+    <x:row r="459">
+      <x:c r="G459" s="57"/>
+      <x:c r="H459"/>
+      <x:c r="I459"/>
+      <x:c r="J459"/>
+      <x:c r="K459" s="64"/>
+    </x:row>
+    <x:row r="460">
+      <x:c r="G460" s="57"/>
+      <x:c r="H460"/>
+      <x:c r="I460"/>
+      <x:c r="J460"/>
+      <x:c r="K460" s="64"/>
+    </x:row>
+    <x:row r="461">
+      <x:c r="G461" s="57"/>
+      <x:c r="H461"/>
+      <x:c r="I461"/>
+      <x:c r="J461"/>
+      <x:c r="K461" s="64"/>
+    </x:row>
+    <x:row r="462">
+      <x:c r="G462" s="57"/>
+      <x:c r="H462"/>
+      <x:c r="I462"/>
+      <x:c r="J462"/>
+      <x:c r="K462" s="64"/>
+    </x:row>
+    <x:row r="463">
+      <x:c r="G463" s="57"/>
+      <x:c r="H463"/>
+      <x:c r="I463"/>
+      <x:c r="J463"/>
+      <x:c r="K463" s="64"/>
+    </x:row>
+    <x:row r="464">
+      <x:c r="G464" s="57"/>
+      <x:c r="H464"/>
+      <x:c r="I464"/>
+      <x:c r="J464"/>
+      <x:c r="K464" s="64"/>
+    </x:row>
+    <x:row r="465">
+      <x:c r="G465" s="57"/>
+      <x:c r="H465"/>
+      <x:c r="I465"/>
+      <x:c r="J465"/>
+      <x:c r="K465" s="64"/>
+    </x:row>
+    <x:row r="466">
+      <x:c r="G466" s="57"/>
+      <x:c r="H466"/>
+      <x:c r="I466"/>
+      <x:c r="J466"/>
+      <x:c r="K466" s="64"/>
+    </x:row>
+    <x:row r="467">
+      <x:c r="G467" s="57"/>
+      <x:c r="H467"/>
+      <x:c r="I467"/>
+      <x:c r="J467"/>
+      <x:c r="K467" s="64"/>
+    </x:row>
+    <x:row r="468">
+      <x:c r="G468" s="57"/>
+      <x:c r="H468"/>
+      <x:c r="I468"/>
+      <x:c r="J468"/>
+      <x:c r="K468" s="64"/>
+    </x:row>
+    <x:row r="469">
+      <x:c r="G469" s="57"/>
+      <x:c r="H469"/>
+      <x:c r="I469"/>
+      <x:c r="J469"/>
+      <x:c r="K469" s="64"/>
+    </x:row>
+    <x:row r="470">
+      <x:c r="G470" s="57"/>
+      <x:c r="H470"/>
+      <x:c r="I470"/>
+      <x:c r="J470"/>
+      <x:c r="K470" s="64"/>
+    </x:row>
+    <x:row r="471">
+      <x:c r="G471" s="57"/>
+      <x:c r="H471"/>
+      <x:c r="I471"/>
+      <x:c r="J471"/>
+      <x:c r="K471" s="64"/>
+    </x:row>
+    <x:row r="472">
+      <x:c r="G472" s="57"/>
+      <x:c r="H472"/>
+      <x:c r="I472"/>
+      <x:c r="J472"/>
+      <x:c r="K472" s="64"/>
+    </x:row>
+    <x:row r="473">
+      <x:c r="G473" s="57"/>
+      <x:c r="H473"/>
+      <x:c r="I473"/>
+      <x:c r="J473"/>
+      <x:c r="K473" s="64"/>
+    </x:row>
+    <x:row r="474">
+      <x:c r="G474" s="57"/>
+      <x:c r="H474"/>
+      <x:c r="I474"/>
+      <x:c r="J474"/>
+      <x:c r="K474" s="64"/>
+    </x:row>
+    <x:row r="475">
+      <x:c r="G475" s="57"/>
+      <x:c r="H475"/>
+      <x:c r="I475"/>
+      <x:c r="J475"/>
+      <x:c r="K475" s="64"/>
+    </x:row>
+    <x:row r="476">
+      <x:c r="G476" s="57"/>
+      <x:c r="H476"/>
+      <x:c r="I476"/>
+      <x:c r="J476"/>
+      <x:c r="K476" s="64"/>
+    </x:row>
+    <x:row r="477">
+      <x:c r="G477" s="57"/>
+      <x:c r="H477"/>
+      <x:c r="I477"/>
+      <x:c r="J477"/>
+      <x:c r="K477" s="64"/>
+    </x:row>
+    <x:row r="478">
+      <x:c r="G478" s="57"/>
+      <x:c r="H478"/>
+      <x:c r="I478"/>
+      <x:c r="J478"/>
+      <x:c r="K478" s="64"/>
+    </x:row>
+    <x:row r="479">
+      <x:c r="G479" s="57"/>
+      <x:c r="H479"/>
+      <x:c r="I479"/>
+      <x:c r="J479"/>
+      <x:c r="K479" s="64"/>
+    </x:row>
+    <x:row r="480">
+      <x:c r="G480" s="57"/>
+      <x:c r="H480"/>
+      <x:c r="I480"/>
+      <x:c r="J480"/>
+      <x:c r="K480" s="64"/>
+    </x:row>
+    <x:row r="481">
+      <x:c r="G481" s="57"/>
+      <x:c r="H481"/>
+      <x:c r="I481"/>
+      <x:c r="J481"/>
+      <x:c r="K481" s="64"/>
+    </x:row>
+    <x:row r="482">
+      <x:c r="G482" s="57"/>
+      <x:c r="H482"/>
+      <x:c r="I482"/>
+      <x:c r="J482"/>
+      <x:c r="K482" s="64"/>
+    </x:row>
+    <x:row r="483">
+      <x:c r="G483" s="57"/>
+      <x:c r="H483"/>
+      <x:c r="I483"/>
+      <x:c r="J483"/>
+      <x:c r="K483" s="64"/>
+    </x:row>
+    <x:row r="484">
+      <x:c r="G484" s="57"/>
+      <x:c r="H484"/>
+      <x:c r="I484"/>
+      <x:c r="J484"/>
+      <x:c r="K484" s="64"/>
+    </x:row>
+    <x:row r="485">
+      <x:c r="G485" s="57"/>
+      <x:c r="H485"/>
+      <x:c r="I485"/>
+      <x:c r="J485"/>
+      <x:c r="K485" s="64"/>
+    </x:row>
+    <x:row r="486">
+      <x:c r="G486" s="57"/>
+      <x:c r="H486"/>
+      <x:c r="I486"/>
+      <x:c r="J486"/>
+      <x:c r="K486" s="64"/>
+    </x:row>
+    <x:row r="487">
+      <x:c r="G487" s="57"/>
+      <x:c r="H487"/>
+      <x:c r="I487"/>
+      <x:c r="J487"/>
+      <x:c r="K487" s="64"/>
+    </x:row>
+    <x:row r="488">
+      <x:c r="G488" s="57"/>
+      <x:c r="H488"/>
+      <x:c r="I488"/>
+      <x:c r="J488"/>
+      <x:c r="K488" s="64"/>
+    </x:row>
+    <x:row r="489">
+      <x:c r="G489" s="57"/>
+      <x:c r="H489"/>
+      <x:c r="I489"/>
+      <x:c r="J489"/>
+      <x:c r="K489" s="64"/>
+    </x:row>
+    <x:row r="490">
+      <x:c r="G490" s="57"/>
+      <x:c r="H490"/>
+      <x:c r="I490"/>
+      <x:c r="J490"/>
+      <x:c r="K490" s="64"/>
+    </x:row>
+    <x:row r="491">
+      <x:c r="G491" s="57"/>
+      <x:c r="H491"/>
+      <x:c r="I491"/>
+      <x:c r="J491"/>
+      <x:c r="K491" s="64"/>
+    </x:row>
+    <x:row r="492">
+      <x:c r="G492" s="57"/>
+      <x:c r="H492"/>
+      <x:c r="I492"/>
+      <x:c r="J492"/>
+      <x:c r="K492" s="64"/>
+    </x:row>
+    <x:row r="493">
+      <x:c r="G493" s="57"/>
+      <x:c r="H493"/>
+      <x:c r="I493"/>
+      <x:c r="J493"/>
+      <x:c r="K493" s="64"/>
+    </x:row>
+    <x:row r="494">
+      <x:c r="G494" s="57"/>
+      <x:c r="H494"/>
+      <x:c r="I494"/>
+      <x:c r="J494"/>
+      <x:c r="K494" s="64"/>
+    </x:row>
+    <x:row r="495">
+      <x:c r="G495" s="57"/>
+      <x:c r="H495"/>
+      <x:c r="I495"/>
+      <x:c r="J495"/>
+      <x:c r="K495" s="64"/>
+    </x:row>
+    <x:row r="496">
+      <x:c r="G496" s="57"/>
+      <x:c r="H496"/>
+      <x:c r="I496"/>
+      <x:c r="J496"/>
+      <x:c r="K496" s="64"/>
+    </x:row>
+    <x:row r="497">
+      <x:c r="G497" s="57"/>
+      <x:c r="H497"/>
+      <x:c r="I497"/>
+      <x:c r="J497"/>
+      <x:c r="K497" s="64"/>
+    </x:row>
+    <x:row r="498">
+      <x:c r="G498" s="57"/>
+      <x:c r="H498"/>
+      <x:c r="I498"/>
+      <x:c r="J498"/>
+      <x:c r="K498" s="64"/>
+    </x:row>
+    <x:row r="499">
+      <x:c r="G499" s="57"/>
+      <x:c r="H499"/>
+      <x:c r="I499"/>
+      <x:c r="J499"/>
+      <x:c r="K499" s="64"/>
+    </x:row>
+    <x:row r="500">
+      <x:c r="G500" s="57"/>
+      <x:c r="H500"/>
+      <x:c r="I500"/>
+      <x:c r="J500"/>
+      <x:c r="K500" s="64"/>
+    </x:row>
+    <x:row r="501">
+      <x:c r="G501" s="57"/>
+      <x:c r="H501"/>
+      <x:c r="I501"/>
+      <x:c r="J501"/>
+      <x:c r="K501" s="65"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B101">
       <x:formula1>"student,faculty,school personnel"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G2:G501">
+      <x:formula1>"Male,Female,Other"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1757,25 +4744,29 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="68" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="24" t="str">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="66" t="str">
         <x:v>CLINiQ Patient Account Import Guide</x:v>
       </x:c>
-      <x:c r="B1" s="24"/>
+      <x:c r="B1" s="66"/>
       <x:c r="C1" s="24"/>
       <x:c r="D1" s="24"/>
       <x:c r="E1" s="24"/>
       <x:c r="F1" s="24"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="27" t="str">
+      <x:c r="A3" s="71" t="str">
         <x:v>Rule</x:v>
       </x:c>
-      <x:c r="B3" s="28" t="str">
+      <x:c r="B3" s="72" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
@@ -1821,51 +4812,55 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="36" t="str">
+        <x:v>Sex</x:v>
+      </x:c>
+      <x:c r="B9" s="36" t="str">
+        <x:v>Required. Use Male, Female, or Other.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="36" t="str">
         <x:v>Student details</x:v>
       </x:c>
-      <x:c r="B9" s="36" t="str">
+      <x:c r="B10" s="36" t="str">
         <x:v>Use an active Program Code (BSIT, BSCS, BSBA, BSA, BSED, BEED, or BSN), Year Level 1 to 4, and Section Code A to E. Program, year level, and section are stored separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="36" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="36" t="str">
         <x:v>Faculty details</x:v>
       </x:c>
-      <x:c r="B10" s="36" t="str">
+      <x:c r="B11" s="36" t="str">
         <x:v>Use an active Department Code (CCS, CBA, COE, CAS, CON, or UHS), Employment Type (Full-time or Part-time), and Title (for example DIT or MIT).</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="37" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="33" t="str">
         <x:v>School personnel details</x:v>
       </x:c>
-      <x:c r="B11" s="37" t="str">
+      <x:c r="B12" s="33" t="str">
         <x:v>Use an active Department Code (CCS, CBA, COE, CAS, CON, or UHS), Employment Type, and Position.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="51" t="str">
-        <x:v>Passwords are generated by CLINiQ after import using the last three ID digits repeated twice. Do not add passwords to this workbook.</x:v>
-      </x:c>
+      <x:c r="A13" s="51"/>
       <x:c r="B13" s="52"/>
       <x:c r="C13" s="52"/>
       <x:c r="D13" s="52"/>
       <x:c r="E13" s="52"/>
       <x:c r="F13" s="53"/>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="54"/>
-      <x:c r="B14" s="55"/>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="69" t="str">
+        <x:v>Passwords are generated by CLINiQ after import using the last three ID digits repeated twice. Do not add passwords to this workbook.</x:v>
+      </x:c>
+      <x:c r="B14" s="70"/>
       <x:c r="C14" s="55"/>
       <x:c r="D14" s="55"/>
       <x:c r="E14" s="55"/>
       <x:c r="F14" s="56"/>
     </x:row>
   </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A13:F14"/>
-  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>